<commit_message>
chore: cập nhật BCTC đầy đủ 2026-10-28
</commit_message>
<xml_diff>
--- a/financials/MBB/MBB.xlsx
+++ b/financials/MBB/MBB.xlsx
@@ -11,6 +11,8 @@
     <sheet name="income_statement" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="cash_flow" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="chi_so_tai_chinh" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Dự báo tăng trưởng" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Hiệu quả thực hiện kế hoạch" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,22 +21,18 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="#,##0;(#,##0);&quot;-&quot;"/>
-    <numFmt numFmtId="165" formatCode="0.0%"/>
-    <numFmt numFmtId="166" formatCode="0.00&quot;x&quot;"/>
-    <numFmt numFmtId="167" formatCode="#,##0 &quot;ngày&quot;"/>
+    <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="166" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
     <font>
       <name val="Tahoma"/>
@@ -47,48 +45,82 @@
     </font>
     <font>
       <name val="Tahoma"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="14"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Tahoma"/>
-      <b val="1"/>
-      <sz val="11"/>
+      <family val="2"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Tahoma"/>
-      <b val="1"/>
+      <family val="2"/>
+      <color rgb="FF000000"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Tahoma"/>
-      <b val="1"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Tahoma"/>
+      <family val="2"/>
       <i val="1"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Tahoma"/>
-      <b val="1"/>
+      <family val="2"/>
+      <color rgb="FF008000"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Tahoma"/>
+      <family val="2"/>
       <i val="1"/>
-      <color rgb="00808080"/>
+      <color rgb="FF808080"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Tahoma"/>
-      <color rgb="00000000"/>
+      <family val="2"/>
+      <color rgb="FF7030A0"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Tahoma"/>
-      <color rgb="00008000"/>
+      <family val="2"/>
+      <i val="1"/>
+      <color rgb="FF7030A0"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Tahoma"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FF008000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Tahoma"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FF7030A0"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Tahoma"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color theme="1"/>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -102,7 +134,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9E1F2"/>
+        <fgColor theme="5" tint="0.7999816888943144"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.7999816888943144"/>
+        <bgColor rgb="FFF7CAAC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.7999816888943144"/>
+        <bgColor rgb="FFFBE4D5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9E1F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -113,12 +163,6 @@
       <top/>
       <bottom/>
       <diagonal/>
-    </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
     </border>
     <border>
       <left style="thin">
@@ -134,38 +178,99 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="5" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="6" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="6" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="6" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="6" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="8" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="9" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="11" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="12" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="13" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="43" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="41" fontId="6" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="10" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="10" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="43" fontId="10" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="2">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="9"/>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -5803,1791 +5908,2534 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I51"/>
+  <dimension ref="A1:J62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="60" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="23" customWidth="1" min="8" max="8"/>
-    <col width="23" customWidth="1" min="9" max="9"/>
-    <col width="3" customWidth="1" min="10" max="10"/>
+    <col width="47.875" customWidth="1" min="1" max="1"/>
+    <col width="17.125" customWidth="1" min="2" max="2"/>
+    <col width="18.125" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>CHỈ SỐ TÀI CHÍNH — MBB</t>
-        </is>
+          <t>Chỉ tiêu</t>
+        </is>
+      </c>
+      <c r="B1" s="6">
+        <f>balance_sheet!B1</f>
+        <v/>
+      </c>
+      <c r="C1" s="6">
+        <f>balance_sheet!C1</f>
+        <v/>
+      </c>
+      <c r="D1" s="6">
+        <f>balance_sheet!D1</f>
+        <v/>
+      </c>
+      <c r="E1" s="6">
+        <f>balance_sheet!E1</f>
+        <v/>
+      </c>
+      <c r="F1" s="6">
+        <f>balance_sheet!F1</f>
+        <v/>
+      </c>
+      <c r="G1" s="6">
+        <f>balance_sheet!G1</f>
+        <v/>
+      </c>
+      <c r="H1" s="6">
+        <f>balance_sheet!H1</f>
+        <v/>
+      </c>
+      <c r="I1" s="6">
+        <f>balance_sheet!I1</f>
+        <v/>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>I. CHỈ SỐ TÀI CHÍNH</t>
-        </is>
-      </c>
-      <c r="B2" s="7" t="n"/>
-      <c r="C2" s="7" t="n"/>
-      <c r="D2" s="7" t="n"/>
-      <c r="E2" s="7" t="n"/>
-      <c r="F2" s="7" t="n"/>
-      <c r="G2" s="7" t="n"/>
-      <c r="H2" s="7" t="n"/>
-      <c r="I2" s="7" t="n"/>
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>ROE</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="n"/>
+      <c r="C2" s="9">
+        <f>IFERROR(C$61/AVERAGE(B$49,C$49),"n/a")</f>
+        <v/>
+      </c>
+      <c r="D2" s="9">
+        <f>IFERROR(D$61/AVERAGE(C$49,D$49),"n/a")</f>
+        <v/>
+      </c>
+      <c r="E2" s="9">
+        <f>IFERROR(E$61/AVERAGE(D$49,E$49),"n/a")</f>
+        <v/>
+      </c>
+      <c r="F2" s="9">
+        <f>IFERROR(F$61/AVERAGE(E$49,F$49),"n/a")</f>
+        <v/>
+      </c>
+      <c r="G2" s="9">
+        <f>IFERROR(G$61/AVERAGE(F$49,G$49),"n/a")</f>
+        <v/>
+      </c>
+      <c r="H2" s="9">
+        <f>IFERROR(H$61/AVERAGE(G$49,H$49),"n/a")</f>
+        <v/>
+      </c>
+      <c r="I2" s="9">
+        <f>IFERROR(I$61/AVERAGE(H$49,I$49),"n/a")</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Tăng trưởng LNST</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="n"/>
+      <c r="C3" s="10">
+        <f>IFERROR((C$61-B$61)/ABS(B$61),"n/a")</f>
+        <v/>
+      </c>
+      <c r="D3" s="10">
+        <f>IFERROR((D$61-C$61)/ABS(C$61),"n/a")</f>
+        <v/>
+      </c>
+      <c r="E3" s="10">
+        <f>IFERROR((E$61-D$61)/ABS(D$61),"n/a")</f>
+        <v/>
+      </c>
+      <c r="F3" s="10">
+        <f>IFERROR((F$61-E$61)/ABS(E$61),"n/a")</f>
+        <v/>
+      </c>
+      <c r="G3" s="10">
+        <f>IFERROR((G$61-F$61)/ABS(F$61),"n/a")</f>
+        <v/>
+      </c>
+      <c r="H3" s="10">
+        <f>IFERROR((H$61-G$61)/ABS(G$61),"n/a")</f>
+        <v/>
+      </c>
+      <c r="I3" s="10">
+        <f>IFERROR((I$61-H$61)/ABS(H$61),"n/a")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Tăng trưởng thu nhập hoạt động</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="n"/>
+      <c r="C4" s="11">
+        <f>IFERROR((C$55-B$55)/ABS(B$55),"n/a")</f>
+        <v/>
+      </c>
+      <c r="D4" s="11">
+        <f>IFERROR((D$55-C$55)/ABS(C$55),"n/a")</f>
+        <v/>
+      </c>
+      <c r="E4" s="11">
+        <f>IFERROR((E$55-D$55)/ABS(D$55),"n/a")</f>
+        <v/>
+      </c>
+      <c r="F4" s="11">
+        <f>IFERROR((F$55-E$55)/ABS(E$55),"n/a")</f>
+        <v/>
+      </c>
+      <c r="G4" s="11">
+        <f>IFERROR((G$55-F$55)/ABS(F$55),"n/a")</f>
+        <v/>
+      </c>
+      <c r="H4" s="11">
+        <f>IFERROR((H$55-G$55)/ABS(G$55),"n/a")</f>
+        <v/>
+      </c>
+      <c r="I4" s="11">
+        <f>IFERROR((I$55-H$55)/ABS(H$55),"n/a")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>% Dư nợ cho vay kinh doanh BĐS</t>
+        </is>
+      </c>
+      <c r="B5" s="8">
+        <f>IFERROR(B$36/#REF!,"n/a")</f>
+        <v/>
+      </c>
+      <c r="C5" s="8">
+        <f>IFERROR(C$36/#REF!,"n/a")</f>
+        <v/>
+      </c>
+      <c r="D5" s="8">
+        <f>IFERROR(D$36/#REF!,"n/a")</f>
+        <v/>
+      </c>
+      <c r="E5" s="8">
+        <f>IFERROR(E$36/#REF!,"n/a")</f>
+        <v/>
+      </c>
+      <c r="F5" s="8">
+        <f>IFERROR(F$36/#REF!,"n/a")</f>
+        <v/>
+      </c>
+      <c r="G5" s="8">
+        <f>IFERROR(G$36/#REF!,"n/a")</f>
+        <v/>
+      </c>
+      <c r="H5" s="8">
+        <f>IFERROR(H$36/#REF!,"n/a")</f>
+        <v/>
+      </c>
+      <c r="I5" s="8">
+        <f>IFERROR(I$36/#REF!,"n/a")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>NIM</t>
+        </is>
+      </c>
+      <c r="B6" s="8">
+        <f>IFERROR(B$55/AVERAGE(B$42,A42),"n/a")</f>
+        <v/>
+      </c>
+      <c r="C6" s="8">
+        <f>IFERROR(C$55/AVERAGE(C$42,B42),"n/a")</f>
+        <v/>
+      </c>
+      <c r="D6" s="8">
+        <f>IFERROR(D$55/AVERAGE(D$42,C42),"n/a")</f>
+        <v/>
+      </c>
+      <c r="E6" s="8">
+        <f>IFERROR(E$55/AVERAGE(E$42,D42),"n/a")</f>
+        <v/>
+      </c>
+      <c r="F6" s="8">
+        <f>IFERROR(F$55/AVERAGE(F$42,E42),"n/a")</f>
+        <v/>
+      </c>
+      <c r="G6" s="8">
+        <f>IFERROR(G$55/AVERAGE(G$42,F42),"n/a")</f>
+        <v/>
+      </c>
+      <c r="H6" s="8">
+        <f>IFERROR(H$55/AVERAGE(H$42,G42),"n/a")</f>
+        <v/>
+      </c>
+      <c r="I6" s="8">
+        <f>IFERROR(I$55/AVERAGE(I$42,H42),"n/a")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>CASA</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="n"/>
+      <c r="C7" s="8" t="n"/>
+      <c r="D7" s="8" t="n"/>
+      <c r="E7" s="8">
+        <f>IFERROR((D$45+E$45+D$48+E$48)/(D$44+E$44),"n/a")</f>
+        <v/>
+      </c>
+      <c r="F7" s="8">
+        <f>IFERROR((E$45+F$45+E$48+F$48)/(E$44+F$44),"n/a")</f>
+        <v/>
+      </c>
+      <c r="G7" s="8">
+        <f>IFERROR((F$45+G$45+F$48+G$48)/(F$44+G$44),"n/a")</f>
+        <v/>
+      </c>
+      <c r="H7" s="8">
+        <f>IFERROR((G$45+H$45+G$48+H$48)/(G$44+H$44),"n/a")</f>
+        <v/>
+      </c>
+      <c r="I7" s="8">
+        <f>IFERROR((H$45+I$45+H$48+I$48)/(H$44+I$44),"n/a")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>NPL</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="n"/>
+      <c r="C8" s="8" t="n"/>
+      <c r="D8" s="8" t="n"/>
+      <c r="E8" s="8">
+        <f>IFERROR((E$35/#REF!),"n/a")</f>
+        <v/>
+      </c>
+      <c r="F8" s="8">
+        <f>IFERROR((F$35/#REF!),"n/a")</f>
+        <v/>
+      </c>
+      <c r="G8" s="8">
+        <f>IFERROR((G$35/#REF!),"n/a")</f>
+        <v/>
+      </c>
+      <c r="H8" s="8">
+        <f>IFERROR((H$35/#REF!),"n/a")</f>
+        <v/>
+      </c>
+      <c r="I8" s="8">
+        <f>IFERROR((I$35/#REF!),"n/a")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>COF</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="n"/>
+      <c r="C9" s="13">
+        <f>IFERROR(ABS(C$54)/AVERAGE(C$42,B42),"n/a")</f>
+        <v/>
+      </c>
+      <c r="D9" s="13">
+        <f>IFERROR(ABS(D$54)/AVERAGE(D$42,C42),"n/a")</f>
+        <v/>
+      </c>
+      <c r="E9" s="13">
+        <f>IFERROR(ABS(E$54)/AVERAGE(E$42,D42),"n/a")</f>
+        <v/>
+      </c>
+      <c r="F9" s="13">
+        <f>IFERROR(ABS(F$54)/AVERAGE(F$42,E42),"n/a")</f>
+        <v/>
+      </c>
+      <c r="G9" s="13">
+        <f>IFERROR(ABS(G$54)/AVERAGE(G$42,F42),"n/a")</f>
+        <v/>
+      </c>
+      <c r="H9" s="13">
+        <f>IFERROR(ABS(H$54)/AVERAGE(H$42,G42),"n/a")</f>
+        <v/>
+      </c>
+      <c r="I9" s="13">
+        <f>IFERROR(ABS(I$54)/AVERAGE(I$42,H42),"n/a")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>LLR</t>
+        </is>
+      </c>
+      <c r="B10" s="8">
+        <f>IFERROR(ABS(B$37)/B$35,"n/a")</f>
+        <v/>
+      </c>
+      <c r="C10" s="8">
+        <f>IFERROR(ABS(C$37)/C$35,"n/a")</f>
+        <v/>
+      </c>
+      <c r="D10" s="8">
+        <f>IFERROR(ABS(D$37)/D$35,"n/a")</f>
+        <v/>
+      </c>
+      <c r="E10" s="8">
+        <f>IFERROR(ABS(E$37)/E$35,"n/a")</f>
+        <v/>
+      </c>
+      <c r="F10" s="8">
+        <f>IFERROR(ABS(F$37)/F$35,"n/a")</f>
+        <v/>
+      </c>
+      <c r="G10" s="8">
+        <f>IFERROR(ABS(G$37)/G$35,"n/a")</f>
+        <v/>
+      </c>
+      <c r="H10" s="8">
+        <f>IFERROR(ABS(H$37)/H$35,"n/a")</f>
+        <v/>
+      </c>
+      <c r="I10" s="8">
+        <f>IFERROR(ABS(I$37)/I$35,"n/a")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>CAR</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="n"/>
+      <c r="C11" s="8" t="n"/>
+      <c r="D11" s="8" t="n"/>
+      <c r="E11" s="8" t="n"/>
+      <c r="F11" s="8" t="n"/>
+      <c r="G11" s="8" t="n"/>
+      <c r="H11" s="8" t="n"/>
+      <c r="I11" s="8" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>LDR</t>
+        </is>
+      </c>
+      <c r="B12" s="8">
+        <f>IFERROR(B$29/B$44,"n/a")</f>
+        <v/>
+      </c>
+      <c r="C12" s="8">
+        <f>IFERROR(C$29/C$44,"n/a")</f>
+        <v/>
+      </c>
+      <c r="D12" s="8">
+        <f>IFERROR(D$29/D$44,"n/a")</f>
+        <v/>
+      </c>
+      <c r="E12" s="8">
+        <f>IFERROR(E$29/E$44,"n/a")</f>
+        <v/>
+      </c>
+      <c r="F12" s="8">
+        <f>IFERROR(F$29/F$44,"n/a")</f>
+        <v/>
+      </c>
+      <c r="G12" s="8">
+        <f>IFERROR(G$29/G$44,"n/a")</f>
+        <v/>
+      </c>
+      <c r="H12" s="8">
+        <f>IFERROR(H$29/H$44,"n/a")</f>
+        <v/>
+      </c>
+      <c r="I12" s="8">
+        <f>IFERROR(I$29/I$44,"n/a")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Tăng trưởng vốn huy động</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="n"/>
+      <c r="C13" s="8">
+        <f>IFERROR((C$44-B$44)/ABS(B$44),"n/a")</f>
+        <v/>
+      </c>
+      <c r="D13" s="8">
+        <f>IFERROR((D$44-C$44)/ABS(C$44),"n/a")</f>
+        <v/>
+      </c>
+      <c r="E13" s="8">
+        <f>IFERROR((E$44-D$44)/ABS(D$44),"n/a")</f>
+        <v/>
+      </c>
+      <c r="F13" s="8">
+        <f>IFERROR((F$44-E$44)/ABS(E$44),"n/a")</f>
+        <v/>
+      </c>
+      <c r="G13" s="8">
+        <f>IFERROR((G$44-F$44)/ABS(F$44),"n/a")</f>
+        <v/>
+      </c>
+      <c r="H13" s="8">
+        <f>IFERROR((H$44-G$44)/ABS(G$44),"n/a")</f>
+        <v/>
+      </c>
+      <c r="I13" s="8">
+        <f>IFERROR((I$44-H$44)/ABS(H$44),"n/a")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Tăng trưởng tín dụng</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="n"/>
+      <c r="C14" s="8">
+        <f>IFERROR((C$29-B$29)/ABS(B$29),"n/a")</f>
+        <v/>
+      </c>
+      <c r="D14" s="8">
+        <f>IFERROR((D$29-C$29)/ABS(C$29),"n/a")</f>
+        <v/>
+      </c>
+      <c r="E14" s="8">
+        <f>IFERROR((E$29-D$29)/ABS(D$29),"n/a")</f>
+        <v/>
+      </c>
+      <c r="F14" s="8">
+        <f>IFERROR((F$29-E$29)/ABS(E$29),"n/a")</f>
+        <v/>
+      </c>
+      <c r="G14" s="8">
+        <f>IFERROR((G$29-F$29)/ABS(F$29),"n/a")</f>
+        <v/>
+      </c>
+      <c r="H14" s="8">
+        <f>IFERROR((H$29-G$29)/ABS(G$29),"n/a")</f>
+        <v/>
+      </c>
+      <c r="I14" s="8">
+        <f>IFERROR((I$29-H$29)/ABS(H$29),"n/a")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>CIR</t>
+        </is>
+      </c>
+      <c r="B15" s="8">
+        <f>IFERROR(ABS(B$58)/B$57,"n/a")</f>
+        <v/>
+      </c>
+      <c r="C15" s="8">
+        <f>IFERROR(ABS(C$58)/C$57,"n/a")</f>
+        <v/>
+      </c>
+      <c r="D15" s="8">
+        <f>IFERROR(ABS(D$58)/D$57,"n/a")</f>
+        <v/>
+      </c>
+      <c r="E15" s="8">
+        <f>IFERROR(ABS(E$58)/E$57,"n/a")</f>
+        <v/>
+      </c>
+      <c r="F15" s="8">
+        <f>IFERROR(ABS(F$58)/F$57,"n/a")</f>
+        <v/>
+      </c>
+      <c r="G15" s="8">
+        <f>IFERROR(ABS(G$58)/G$57,"n/a")</f>
+        <v/>
+      </c>
+      <c r="H15" s="8">
+        <f>IFERROR(ABS(H$58)/H$57,"n/a")</f>
+        <v/>
+      </c>
+      <c r="I15" s="8">
+        <f>IFERROR(ABS(I$58)/I$57,"n/a")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>VCSH/Tổng tài sản</t>
+        </is>
+      </c>
+      <c r="B16" s="13">
+        <f>IFERROR(B$49/B$24,"n/a")</f>
+        <v/>
+      </c>
+      <c r="C16" s="13">
+        <f>IFERROR(C$49/C$24,"n/a")</f>
+        <v/>
+      </c>
+      <c r="D16" s="13">
+        <f>IFERROR(D$49/D$24,"n/a")</f>
+        <v/>
+      </c>
+      <c r="E16" s="13">
+        <f>IFERROR(E$49/E$24,"n/a")</f>
+        <v/>
+      </c>
+      <c r="F16" s="13">
+        <f>IFERROR(F$49/F$24,"n/a")</f>
+        <v/>
+      </c>
+      <c r="G16" s="13">
+        <f>IFERROR(G$49/G$24,"n/a")</f>
+        <v/>
+      </c>
+      <c r="H16" s="13">
+        <f>IFERROR(H$49/H$24,"n/a")</f>
+        <v/>
+      </c>
+      <c r="I16" s="13">
+        <f>IFERROR(I$49/I$24,"n/a")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>Tỷ lệ lãi và phí phải thu/Thu nhập lãi</t>
+        </is>
+      </c>
+      <c r="B17" s="13">
+        <f>IFERROR(B59/B$53,"n/a")</f>
+        <v/>
+      </c>
+      <c r="C17" s="13">
+        <f>IFERROR(C59/C$53,"n/a")</f>
+        <v/>
+      </c>
+      <c r="D17" s="13">
+        <f>IFERROR(D59/D$53,"n/a")</f>
+        <v/>
+      </c>
+      <c r="E17" s="13">
+        <f>IFERROR(E59/E$53,"n/a")</f>
+        <v/>
+      </c>
+      <c r="F17" s="13">
+        <f>IFERROR(F59/F$53,"n/a")</f>
+        <v/>
+      </c>
+      <c r="G17" s="13">
+        <f>IFERROR(G59/G$53,"n/a")</f>
+        <v/>
+      </c>
+      <c r="H17" s="13">
+        <f>IFERROR(H59/H$53,"n/a")</f>
+        <v/>
+      </c>
+      <c r="I17" s="13">
+        <f>IFERROR(I59/I$53,"n/a")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>Thu nhập ngoài lãi/Thu nhập hoạt động</t>
+        </is>
+      </c>
+      <c r="B18" s="8">
+        <f>IFERROR(B$56/B$57,"n/a")</f>
+        <v/>
+      </c>
+      <c r="C18" s="8">
+        <f>IFERROR(C$56/C$57,"n/a")</f>
+        <v/>
+      </c>
+      <c r="D18" s="8">
+        <f>IFERROR(D$56/D$57,"n/a")</f>
+        <v/>
+      </c>
+      <c r="E18" s="8">
+        <f>IFERROR(E$56/E$57,"n/a")</f>
+        <v/>
+      </c>
+      <c r="F18" s="8">
+        <f>IFERROR(F$56/F$57,"n/a")</f>
+        <v/>
+      </c>
+      <c r="G18" s="8">
+        <f>IFERROR(G$56/G$57,"n/a")</f>
+        <v/>
+      </c>
+      <c r="H18" s="8">
+        <f>IFERROR(H$56/H$57,"n/a")</f>
+        <v/>
+      </c>
+      <c r="I18" s="8">
+        <f>IFERROR(I$56/I$57,"n/a")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19"/>
+    <row r="20">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>II. DỮ LIỆU TRÍCH XUẤT (tự động dò theo tên khoản mục)</t>
+        </is>
+      </c>
+      <c r="B20" s="15" t="n"/>
+      <c r="C20" s="15" t="n"/>
+      <c r="D20" s="15" t="n"/>
+      <c r="E20" s="15" t="n"/>
+      <c r="F20" s="15" t="n"/>
+      <c r="G20" s="15" t="n"/>
+      <c r="H20" s="15" t="n"/>
+      <c r="I20" s="15" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="16" t="inlineStr">
+        <is>
+          <t>Khoản mục</t>
+        </is>
+      </c>
+      <c r="B21" s="17">
+        <f>balance_sheet!B1</f>
+        <v/>
+      </c>
+      <c r="C21" s="17">
+        <f>balance_sheet!C1</f>
+        <v/>
+      </c>
+      <c r="D21" s="17">
+        <f>balance_sheet!D1</f>
+        <v/>
+      </c>
+      <c r="E21" s="17">
+        <f>balance_sheet!E1</f>
+        <v/>
+      </c>
+      <c r="F21" s="17">
+        <f>balance_sheet!F1</f>
+        <v/>
+      </c>
+      <c r="G21" s="17">
+        <f>balance_sheet!G1</f>
+        <v/>
+      </c>
+      <c r="H21" s="17">
+        <f>balance_sheet!H1</f>
+        <v/>
+      </c>
+      <c r="I21" s="17">
+        <f>balance_sheet!I1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="16" t="inlineStr">
+        <is>
+          <t>CĐKT</t>
+        </is>
+      </c>
+      <c r="B22" s="18" t="n"/>
+      <c r="C22" s="18" t="n"/>
+      <c r="D22" s="18" t="n"/>
+      <c r="E22" s="18" t="n"/>
+      <c r="F22" s="18" t="n"/>
+      <c r="G22" s="18" t="n"/>
+      <c r="H22" s="18" t="n"/>
+      <c r="I22" s="18" t="n"/>
+      <c r="J22" s="19" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="16" t="inlineStr">
+        <is>
+          <t>Tài sản</t>
+        </is>
+      </c>
+      <c r="B23" s="18" t="n"/>
+      <c r="C23" s="18" t="n"/>
+      <c r="D23" s="18" t="n"/>
+      <c r="E23" s="18" t="n"/>
+      <c r="F23" s="18" t="n"/>
+      <c r="G23" s="18" t="n"/>
+      <c r="H23" s="18" t="n"/>
+      <c r="I23" s="18" t="n"/>
+      <c r="J23" s="19" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="20" t="inlineStr">
+        <is>
+          <t>TỔNG TÀI SẢN</t>
+        </is>
+      </c>
+      <c r="B24" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("TỔNG TÀI SẢN",balance_sheet!$A:$A,0),MATCH(B$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C24" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("TỔNG TÀI SẢN",balance_sheet!$A:$A,0),MATCH(C$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D24" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("TỔNG TÀI SẢN",balance_sheet!$A:$A,0),MATCH(D$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E24" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("TỔNG TÀI SẢN",balance_sheet!$A:$A,0),MATCH(E$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="F24" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("TỔNG TÀI SẢN",balance_sheet!$A:$A,0),MATCH(F$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G24" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("TỔNG TÀI SẢN",balance_sheet!$A:$A,0),MATCH(G$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="H24" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("TỔNG TÀI SẢN",balance_sheet!$A:$A,0),MATCH(H$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="I24" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("TỔNG TÀI SẢN",balance_sheet!$A:$A,0),MATCH(I$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J24" s="19" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="20" t="inlineStr">
+        <is>
+          <t>Tiền gửi tại Ngân hàng nhà nước Việt Nam</t>
+        </is>
+      </c>
+      <c r="B25" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Tiền gửi tại Ngân hàng nhà nước Việt Nam",balance_sheet!$A:$A,0),MATCH(B$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C25" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Tiền gửi tại Ngân hàng nhà nước Việt Nam",balance_sheet!$A:$A,0),MATCH(C$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D25" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Tiền gửi tại Ngân hàng nhà nước Việt Nam",balance_sheet!$A:$A,0),MATCH(D$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E25" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Tiền gửi tại Ngân hàng nhà nước Việt Nam",balance_sheet!$A:$A,0),MATCH(E$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="F25" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Tiền gửi tại Ngân hàng nhà nước Việt Nam",balance_sheet!$A:$A,0),MATCH(F$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G25" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Tiền gửi tại Ngân hàng nhà nước Việt Nam",balance_sheet!$A:$A,0),MATCH(G$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="H25" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Tiền gửi tại Ngân hàng nhà nước Việt Nam",balance_sheet!$A:$A,0),MATCH(H$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="I25" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Tiền gửi tại Ngân hàng nhà nước Việt Nam",balance_sheet!$A:$A,0),MATCH(I$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J25" s="19" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="20" t="inlineStr">
+        <is>
+          <t>Tiền gửi tại các TCTD khác và cho vay các TCTD khác</t>
+        </is>
+      </c>
+      <c r="B26" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Tiền gửi tại các TCTD khác và cho vay các TCTD khác",balance_sheet!$A:$A,0),MATCH(B$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C26" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Tiền gửi tại các TCTD khác và cho vay các TCTD khác",balance_sheet!$A:$A,0),MATCH(C$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D26" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Tiền gửi tại các TCTD khác và cho vay các TCTD khác",balance_sheet!$A:$A,0),MATCH(D$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E26" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Tiền gửi tại các TCTD khác và cho vay các TCTD khác",balance_sheet!$A:$A,0),MATCH(E$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="F26" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Tiền gửi tại các TCTD khác và cho vay các TCTD khác",balance_sheet!$A:$A,0),MATCH(F$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G26" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Tiền gửi tại các TCTD khác và cho vay các TCTD khác",balance_sheet!$A:$A,0),MATCH(G$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="H26" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Tiền gửi tại các TCTD khác và cho vay các TCTD khác",balance_sheet!$A:$A,0),MATCH(H$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="I26" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Tiền gửi tại các TCTD khác và cho vay các TCTD khác",balance_sheet!$A:$A,0),MATCH(I$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J26" s="19" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="20" t="inlineStr">
+        <is>
+          <t>Dự phòng rủi ro cho cay các TCTC khác</t>
+        </is>
+      </c>
+      <c r="B27" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Dự phòng rủi ro",balance_sheet!$A:$A,0),MATCH(B$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C27" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Dự phòng rủi ro",balance_sheet!$A:$A,0),MATCH(C$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D27" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Dự phòng rủi ro",balance_sheet!$A:$A,0),MATCH(D$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E27" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Dự phòng rủi ro",balance_sheet!$A:$A,0),MATCH(E$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="F27" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Dự phòng rủi ro",balance_sheet!$A:$A,0),MATCH(F$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G27" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Dự phòng rủi ro",balance_sheet!$A:$A,0),MATCH(G$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="H27" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Dự phòng rủi ro",balance_sheet!$A:$A,0),MATCH(H$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="I27" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Dự phòng rủi ro",balance_sheet!$A:$A,0),MATCH(I$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J27" s="19" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="20" t="inlineStr">
+        <is>
+          <t>Chứng khoán kinh doanh</t>
+        </is>
+      </c>
+      <c r="B28" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Chứng khoán kinh doanh",balance_sheet!$A:$A,0),MATCH(B$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C28" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Chứng khoán kinh doanh",balance_sheet!$A:$A,0),MATCH(C$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D28" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Chứng khoán kinh doanh",balance_sheet!$A:$A,0),MATCH(D$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E28" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Chứng khoán kinh doanh",balance_sheet!$A:$A,0),MATCH(E$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="F28" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Chứng khoán kinh doanh",balance_sheet!$A:$A,0),MATCH(F$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G28" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Chứng khoán kinh doanh",balance_sheet!$A:$A,0),MATCH(G$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="H28" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Chứng khoán kinh doanh",balance_sheet!$A:$A,0),MATCH(H$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="I28" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Chứng khoán kinh doanh",balance_sheet!$A:$A,0),MATCH(I$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J28" s="19" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="20" t="inlineStr">
+        <is>
+          <t>Cho vay khách hàng</t>
+        </is>
+      </c>
+      <c r="B29" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Cho vay khách hàng",balance_sheet!$A:$A,0),MATCH(B$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C29" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Cho vay khách hàng",balance_sheet!$A:$A,0),MATCH(C$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D29" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Cho vay khách hàng",balance_sheet!$A:$A,0),MATCH(D$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E29" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Cho vay khách hàng",balance_sheet!$A:$A,0),MATCH(E$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="F29" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Cho vay khách hàng",balance_sheet!$A:$A,0),MATCH(F$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G29" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Cho vay khách hàng",balance_sheet!$A:$A,0),MATCH(G$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="H29" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Cho vay khách hàng",balance_sheet!$A:$A,0),MATCH(H$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="I29" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Cho vay khách hàng",balance_sheet!$A:$A,0),MATCH(I$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J29" s="19" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="20" t="inlineStr">
+        <is>
+          <t>+ Nợ đủ tiêu chuẩn</t>
+        </is>
+      </c>
+      <c r="B30" s="22" t="n"/>
+      <c r="C30" s="22" t="n"/>
+      <c r="D30" s="22" t="n"/>
+      <c r="E30" s="22" t="n">
+        <v>349223000000000</v>
+      </c>
+      <c r="F30" s="22" t="n">
+        <v>443975000000000</v>
+      </c>
+      <c r="G30" s="22" t="n">
+        <v>587326000000000</v>
+      </c>
+      <c r="H30" s="22" t="n">
+        <v>751876000000000</v>
+      </c>
+      <c r="I30" s="22" t="n">
+        <v>1059782000000000</v>
+      </c>
+      <c r="J30" s="23" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="20" t="inlineStr">
+        <is>
+          <t>+ Nợ cần chú ý</t>
+        </is>
+      </c>
+      <c r="B31" s="22" t="n"/>
+      <c r="C31" s="22" t="n"/>
+      <c r="D31" s="22" t="n"/>
+      <c r="E31" s="22" t="n">
+        <v>3913000000000</v>
+      </c>
+      <c r="F31" s="22" t="n">
+        <v>7809000000000</v>
+      </c>
+      <c r="G31" s="22" t="n">
+        <v>13918000000000</v>
+      </c>
+      <c r="H31" s="22" t="n">
+        <v>12197000000000</v>
+      </c>
+      <c r="I31" s="22" t="n">
+        <v>10210000000000</v>
+      </c>
+      <c r="J31" s="19" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="20" t="inlineStr">
+        <is>
+          <t>+ Nợ dưới tiêu chuẩn</t>
+        </is>
+      </c>
+      <c r="B32" s="22" t="n"/>
+      <c r="C32" s="22" t="n"/>
+      <c r="D32" s="22" t="n"/>
+      <c r="E32" s="22" t="n">
+        <v>1433000000000</v>
+      </c>
+      <c r="F32" s="22" t="n">
+        <v>1517000000000</v>
+      </c>
+      <c r="G32" s="22" t="n">
+        <v>3211000000000</v>
+      </c>
+      <c r="H32" s="22" t="n">
+        <v>3380000000000</v>
+      </c>
+      <c r="I32" s="22" t="n">
+        <v>3276000000000</v>
+      </c>
+      <c r="J32" s="19" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="20" t="inlineStr">
+        <is>
+          <t>+ Nợ nghi ngờ</t>
+        </is>
+      </c>
+      <c r="B33" s="22" t="n"/>
+      <c r="C33" s="22" t="n"/>
+      <c r="D33" s="22" t="n"/>
+      <c r="E33" s="22" t="n">
+        <v>1015000000000</v>
+      </c>
+      <c r="F33" s="22" t="n">
+        <v>1221000000000</v>
+      </c>
+      <c r="G33" s="22" t="n">
+        <v>3704000000000</v>
+      </c>
+      <c r="H33" s="22" t="n">
+        <v>4599000000000</v>
+      </c>
+      <c r="I33" s="22" t="n">
+        <v>4330000000000</v>
+      </c>
+      <c r="J33" s="19" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="20" t="inlineStr">
+        <is>
+          <t>+ Nợ có khả năng mất vốn</t>
+        </is>
+      </c>
+      <c r="B34" s="22" t="n"/>
+      <c r="C34" s="22" t="n"/>
+      <c r="D34" s="22" t="n"/>
+      <c r="E34" s="22" t="n">
+        <v>819000000000</v>
+      </c>
+      <c r="F34" s="22" t="n">
+        <v>2293000000000</v>
+      </c>
+      <c r="G34" s="22" t="n">
+        <v>2890000000000</v>
+      </c>
+      <c r="H34" s="22" t="n">
+        <v>4607000000000</v>
+      </c>
+      <c r="I34" s="22" t="n">
+        <v>6421000000000</v>
+      </c>
+      <c r="J34" s="23" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="24" t="inlineStr">
+        <is>
+          <t>Nợ xấu</t>
+        </is>
+      </c>
+      <c r="B35" s="25">
+        <f>SUM(B32:B34)</f>
+        <v/>
+      </c>
+      <c r="C35" s="25">
+        <f>SUM(C32:C34)</f>
+        <v/>
+      </c>
+      <c r="D35" s="25">
+        <f>SUM(D32:D34)</f>
+        <v/>
+      </c>
+      <c r="E35" s="25">
+        <f>SUM(E32:E34)</f>
+        <v/>
+      </c>
+      <c r="F35" s="25">
+        <f>SUM(F32:F34)</f>
+        <v/>
+      </c>
+      <c r="G35" s="25">
+        <f>SUM(G32:G34)</f>
+        <v/>
+      </c>
+      <c r="H35" s="25">
+        <f>SUM(H32:H34)</f>
+        <v/>
+      </c>
+      <c r="I35" s="25">
+        <f>SUM(I32:I34)</f>
+        <v/>
+      </c>
+      <c r="J35" s="26" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="20" t="inlineStr">
+        <is>
+          <t>Cho vay KDBĐS</t>
+        </is>
+      </c>
+      <c r="B36" s="22" t="n"/>
+      <c r="C36" s="22" t="n"/>
+      <c r="D36" s="22" t="n"/>
+      <c r="E36" s="22" t="n">
+        <v>12632000000000</v>
+      </c>
+      <c r="F36" s="22" t="n">
+        <v>21358000000000</v>
+      </c>
+      <c r="G36" s="22" t="n">
+        <v>43268000000000</v>
+      </c>
+      <c r="H36" s="22" t="n">
+        <v>64141000000000</v>
+      </c>
+      <c r="I36" s="22" t="n">
+        <v>121189000000000</v>
+      </c>
+      <c r="J36" s="19" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="20" t="inlineStr">
+        <is>
+          <t>Dự phòng rủi ro cho vay khách hàng</t>
+        </is>
+      </c>
+      <c r="B37" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Dự phòng rủi ro cho vay khách hàng",balance_sheet!$A:$A,0),MATCH(B$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C37" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Dự phòng rủi ro cho vay khách hàng",balance_sheet!$A:$A,0),MATCH(C$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D37" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Dự phòng rủi ro cho vay khách hàng",balance_sheet!$A:$A,0),MATCH(D$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E37" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Dự phòng rủi ro cho vay khách hàng",balance_sheet!$A:$A,0),MATCH(E$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="F37" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Dự phòng rủi ro cho vay khách hàng",balance_sheet!$A:$A,0),MATCH(F$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G37" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Dự phòng rủi ro cho vay khách hàng",balance_sheet!$A:$A,0),MATCH(G$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="H37" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Dự phòng rủi ro cho vay khách hàng",balance_sheet!$A:$A,0),MATCH(H$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="I37" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Dự phòng rủi ro cho vay khách hàng",balance_sheet!$A:$A,0),MATCH(I$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J37" s="19" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="20" t="inlineStr">
+        <is>
+          <t>Chứng khoán đầu tư</t>
+        </is>
+      </c>
+      <c r="B38" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Chứng khoán đầu tư",balance_sheet!$A:$A,0),MATCH(B$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C38" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Chứng khoán đầu tư",balance_sheet!$A:$A,0),MATCH(C$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D38" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Chứng khoán đầu tư",balance_sheet!$A:$A,0),MATCH(D$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E38" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Chứng khoán đầu tư",balance_sheet!$A:$A,0),MATCH(E$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="F38" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Chứng khoán đầu tư",balance_sheet!$A:$A,0),MATCH(F$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G38" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Chứng khoán đầu tư",balance_sheet!$A:$A,0),MATCH(G$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="H38" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Chứng khoán đầu tư",balance_sheet!$A:$A,0),MATCH(H$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="I38" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Chứng khoán đầu tư",balance_sheet!$A:$A,0),MATCH(I$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J38" s="19" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="20" t="inlineStr">
+        <is>
+          <t>Dự phòng giảm giá chứng khoán đầu tư</t>
+        </is>
+      </c>
+      <c r="B39" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Dự phòng giảm giá chứng khoán đầu tư",balance_sheet!$A:$A,0),MATCH(B$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C39" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Dự phòng giảm giá chứng khoán đầu tư",balance_sheet!$A:$A,0),MATCH(C$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D39" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Dự phòng giảm giá chứng khoán đầu tư",balance_sheet!$A:$A,0),MATCH(D$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E39" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Dự phòng giảm giá chứng khoán đầu tư",balance_sheet!$A:$A,0),MATCH(E$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="F39" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Dự phòng giảm giá chứng khoán đầu tư",balance_sheet!$A:$A,0),MATCH(F$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G39" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Dự phòng giảm giá chứng khoán đầu tư",balance_sheet!$A:$A,0),MATCH(G$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="H39" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Dự phòng giảm giá chứng khoán đầu tư",balance_sheet!$A:$A,0),MATCH(H$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="I39" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Dự phòng giảm giá chứng khoán đầu tư",balance_sheet!$A:$A,0),MATCH(I$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J39" s="19" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="20" t="inlineStr">
+        <is>
+          <t>Góp vốn, đầu tư dài hạn</t>
+        </is>
+      </c>
+      <c r="B40" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Góp vốn, đầu tư dài hạn",balance_sheet!$A:$A,0),MATCH(B$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C40" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Góp vốn, đầu tư dài hạn",balance_sheet!$A:$A,0),MATCH(C$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D40" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Góp vốn, đầu tư dài hạn",balance_sheet!$A:$A,0),MATCH(D$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E40" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Góp vốn, đầu tư dài hạn",balance_sheet!$A:$A,0),MATCH(E$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="F40" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Góp vốn, đầu tư dài hạn",balance_sheet!$A:$A,0),MATCH(F$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G40" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Góp vốn, đầu tư dài hạn",balance_sheet!$A:$A,0),MATCH(G$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="H40" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Góp vốn, đầu tư dài hạn",balance_sheet!$A:$A,0),MATCH(H$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="I40" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Góp vốn, đầu tư dài hạn",balance_sheet!$A:$A,0),MATCH(I$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J40" s="19" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="20" t="inlineStr">
+        <is>
+          <t>Dự phòng giảm giá đầu tư dài hạn</t>
+        </is>
+      </c>
+      <c r="B41" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Dự phòng giảm giá đầu tư dài hạn",balance_sheet!$A:$A,0),MATCH(B$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C41" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Dự phòng giảm giá đầu tư dài hạn",balance_sheet!$A:$A,0),MATCH(C$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D41" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Dự phòng giảm giá đầu tư dài hạn",balance_sheet!$A:$A,0),MATCH(D$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E41" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Dự phòng giảm giá đầu tư dài hạn",balance_sheet!$A:$A,0),MATCH(E$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="F41" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Dự phòng giảm giá đầu tư dài hạn",balance_sheet!$A:$A,0),MATCH(F$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G41" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Dự phòng giảm giá đầu tư dài hạn",balance_sheet!$A:$A,0),MATCH(G$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="H41" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Dự phòng giảm giá đầu tư dài hạn",balance_sheet!$A:$A,0),MATCH(H$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="I41" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Dự phòng giảm giá đầu tư dài hạn",balance_sheet!$A:$A,0),MATCH(I$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J41" s="19" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="20" t="inlineStr">
+        <is>
+          <t>Tài sản sinh lời</t>
+        </is>
+      </c>
+      <c r="B42" s="25">
+        <f>B25+B26-B27+B28+B29+B38-B39+B40-B41</f>
+        <v/>
+      </c>
+      <c r="C42" s="25">
+        <f>C25+C26-C27+C28+C29+C38-C39+C40-C41</f>
+        <v/>
+      </c>
+      <c r="D42" s="25">
+        <f>D25+D26-D27+D28+D29+D38-D39+D40-D41</f>
+        <v/>
+      </c>
+      <c r="E42" s="25">
+        <f>E25+E26-E27+E28+E29+E38-E39+E40-E41</f>
+        <v/>
+      </c>
+      <c r="F42" s="25">
+        <f>F25+F26-F27+F28+F29+F38-F39+F40-F41</f>
+        <v/>
+      </c>
+      <c r="G42" s="25">
+        <f>G25+G26-G27+G28+G29+G38-G39+G40-G41</f>
+        <v/>
+      </c>
+      <c r="H42" s="25">
+        <f>H25+H26-H27+H28+H29+H38-H39+H40-H41</f>
+        <v/>
+      </c>
+      <c r="I42" s="25">
+        <f>I25+I26-I27+I28+I29+I38-I39+I40-I41</f>
+        <v/>
+      </c>
+      <c r="J42" s="19" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="16" t="inlineStr">
+        <is>
+          <t>Nguồn vốn</t>
+        </is>
+      </c>
+      <c r="B43" s="21" t="n"/>
+      <c r="C43" s="21" t="n"/>
+      <c r="D43" s="21" t="n"/>
+      <c r="E43" s="21" t="n"/>
+      <c r="F43" s="21" t="n"/>
+      <c r="G43" s="21" t="n"/>
+      <c r="H43" s="21" t="n"/>
+      <c r="I43" s="21" t="n"/>
+      <c r="J43" s="19" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="20" t="inlineStr">
+        <is>
+          <t>Tiền gửi khách hàng</t>
+        </is>
+      </c>
+      <c r="B44" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Tiền gửi của khách hàng",balance_sheet!$A:$A,0),MATCH(B$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C44" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Tiền gửi của khách hàng",balance_sheet!$A:$A,0),MATCH(C$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D44" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Tiền gửi của khách hàng",balance_sheet!$A:$A,0),MATCH(D$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E44" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Tiền gửi của khách hàng",balance_sheet!$A:$A,0),MATCH(E$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="F44" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Tiền gửi của khách hàng",balance_sheet!$A:$A,0),MATCH(F$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G44" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Tiền gửi của khách hàng",balance_sheet!$A:$A,0),MATCH(G$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="H44" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Tiền gửi của khách hàng",balance_sheet!$A:$A,0),MATCH(H$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="I44" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Tiền gửi của khách hàng",balance_sheet!$A:$A,0),MATCH(I$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J44" s="19" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="20" t="inlineStr">
+        <is>
+          <t>+ Tiền gửi không kỳ hạn</t>
+        </is>
+      </c>
+      <c r="B45" s="22" t="n"/>
+      <c r="C45" s="22" t="n"/>
+      <c r="D45" s="22" t="n"/>
+      <c r="E45" s="22" t="n">
+        <v>171396000000000</v>
+      </c>
+      <c r="F45" s="22" t="n">
+        <v>166972000000000</v>
+      </c>
+      <c r="G45" s="22" t="n">
+        <v>216092000000000</v>
+      </c>
+      <c r="H45" s="22" t="n">
+        <v>271580000000000</v>
+      </c>
+      <c r="I45" s="22" t="n">
+        <v>339353000000000</v>
+      </c>
+      <c r="J45" s="19" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="20" t="inlineStr">
+        <is>
+          <t>+ Tiền gửi có kỳ hạn</t>
+        </is>
+      </c>
+      <c r="B46" s="22" t="n"/>
+      <c r="C46" s="22" t="n"/>
+      <c r="D46" s="22" t="n"/>
+      <c r="E46" s="22" t="n">
+        <v>197180000000000</v>
+      </c>
+      <c r="F46" s="22" t="n">
+        <v>263452000000000</v>
+      </c>
+      <c r="G46" s="22" t="n">
+        <v>339421000000000</v>
+      </c>
+      <c r="H46" s="22" t="n">
+        <v>433477000000000</v>
+      </c>
+      <c r="I46" s="22" t="n">
+        <v>573483000000000</v>
+      </c>
+      <c r="J46" s="19" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="20" t="inlineStr">
+        <is>
+          <t>+ Tiền gửi vốn chuyên dùng</t>
+        </is>
+      </c>
+      <c r="B47" s="22" t="n"/>
+      <c r="C47" s="22" t="n"/>
+      <c r="D47" s="22" t="n"/>
+      <c r="E47" s="22" t="n">
+        <v>4389000000000</v>
+      </c>
+      <c r="F47" s="22" t="n">
+        <v>2827000000000</v>
+      </c>
+      <c r="G47" s="22" t="n">
+        <v>3264000000000</v>
+      </c>
+      <c r="H47" s="22" t="n">
+        <v>1791000000000</v>
+      </c>
+      <c r="I47" s="22" t="n">
+        <v>1226000000000</v>
+      </c>
+      <c r="J47" s="19" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="20" t="inlineStr">
+        <is>
+          <t>+ Tiền ký quỹ</t>
+        </is>
+      </c>
+      <c r="B48" s="22" t="n"/>
+      <c r="C48" s="22" t="n"/>
+      <c r="D48" s="22" t="n"/>
+      <c r="E48" s="22" t="n">
+        <v>11728000000000</v>
+      </c>
+      <c r="F48" s="22" t="n">
+        <v>10355000000000</v>
+      </c>
+      <c r="G48" s="22" t="n">
+        <v>8755000000000</v>
+      </c>
+      <c r="H48" s="22" t="n">
+        <v>7307000000000</v>
+      </c>
+      <c r="I48" s="22" t="n">
+        <v>7307000000000</v>
+      </c>
+      <c r="J48" s="19" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="16" t="inlineStr">
+        <is>
+          <t>VỐN CHỦ SỞ HỮU</t>
+        </is>
+      </c>
+      <c r="B49" s="27">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("VỐN CHỦ SỞ HỮU",balance_sheet!$A:$A,0),MATCH(B$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C49" s="27">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("VỐN CHỦ SỞ HỮU",balance_sheet!$A:$A,0),MATCH(C$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D49" s="27">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("VỐN CHỦ SỞ HỮU",balance_sheet!$A:$A,0),MATCH(D$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E49" s="27">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("VỐN CHỦ SỞ HỮU",balance_sheet!$A:$A,0),MATCH(E$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="F49" s="27">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("VỐN CHỦ SỞ HỮU",balance_sheet!$A:$A,0),MATCH(F$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G49" s="27">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("VỐN CHỦ SỞ HỮU",balance_sheet!$A:$A,0),MATCH(G$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="H49" s="27">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("VỐN CHỦ SỞ HỮU",balance_sheet!$A:$A,0),MATCH(H$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="I49" s="27">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("VỐN CHỦ SỞ HỮU",balance_sheet!$A:$A,0),MATCH(I$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J49" s="27">
+        <f>I49+0.9*J61</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="28" t="inlineStr">
+        <is>
+          <t>Tăng VCSH/LN cty mẹ</t>
+        </is>
+      </c>
+      <c r="B50" s="29" t="n"/>
+      <c r="C50" s="29">
+        <f>(C49-B49)/C61</f>
+        <v/>
+      </c>
+      <c r="D50" s="29">
+        <f>(D49-C49)/D61</f>
+        <v/>
+      </c>
+      <c r="E50" s="29">
+        <f>(E49-D49)/E61</f>
+        <v/>
+      </c>
+      <c r="F50" s="29">
+        <f>(F49-E49)/F61</f>
+        <v/>
+      </c>
+      <c r="G50" s="29">
+        <f>(G49-F49)/G61</f>
+        <v/>
+      </c>
+      <c r="H50" s="29">
+        <f>(H49-G49)/H61</f>
+        <v/>
+      </c>
+      <c r="I50" s="29">
+        <f>(I49-H49)/I61</f>
+        <v/>
+      </c>
+      <c r="J50" s="30" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="16" t="inlineStr">
+        <is>
+          <t>Lợi ích của cổ đông thiểu số</t>
+        </is>
+      </c>
+      <c r="B51" s="27">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Lợi ích của cổ đông thiểu số",balance_sheet!$A:$A,0),MATCH(B$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C51" s="27">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Lợi ích của cổ đông thiểu số",balance_sheet!$A:$A,0),MATCH(C$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D51" s="27">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Lợi ích của cổ đông thiểu số",balance_sheet!$A:$A,0),MATCH(D$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E51" s="27">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Lợi ích của cổ đông thiểu số",balance_sheet!$A:$A,0),MATCH(E$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="F51" s="27">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Lợi ích của cổ đông thiểu số",balance_sheet!$A:$A,0),MATCH(F$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G51" s="27">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Lợi ích của cổ đông thiểu số",balance_sheet!$A:$A,0),MATCH(G$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="H51" s="27">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Lợi ích của cổ đông thiểu số",balance_sheet!$A:$A,0),MATCH(H$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="I51" s="27">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Lợi ích của cổ đông thiểu số",balance_sheet!$A:$A,0),MATCH(I$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J51" s="31" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="16" t="inlineStr">
+        <is>
+          <t>Kết quả hoạt động kinh doanh</t>
+        </is>
+      </c>
+      <c r="B52" s="21" t="n"/>
+      <c r="C52" s="21" t="n"/>
+      <c r="D52" s="21" t="n"/>
+      <c r="E52" s="21" t="n"/>
+      <c r="F52" s="21" t="n"/>
+      <c r="G52" s="21" t="n"/>
+      <c r="H52" s="21" t="n"/>
+      <c r="I52" s="21" t="n"/>
+      <c r="J52" s="19" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="20" t="inlineStr">
+        <is>
+          <t>Thu nhập lãi</t>
+        </is>
+      </c>
+      <c r="B53" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Thu nhập lãi và các khoản thu nhập tương tự",income_statement!$A:$A,0),MATCH(B$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C53" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Thu nhập lãi và các khoản thu nhập tương tự",income_statement!$A:$A,0),MATCH(C$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D53" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Thu nhập lãi và các khoản thu nhập tương tự",income_statement!$A:$A,0),MATCH(D$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E53" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Thu nhập lãi và các khoản thu nhập tương tự",income_statement!$A:$A,0),MATCH(E$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="F53" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Thu nhập lãi và các khoản thu nhập tương tự",income_statement!$A:$A,0),MATCH(F$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G53" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Thu nhập lãi và các khoản thu nhập tương tự",income_statement!$A:$A,0),MATCH(G$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="H53" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Thu nhập lãi và các khoản thu nhập tương tự",income_statement!$A:$A,0),MATCH(H$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="I53" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Thu nhập lãi và các khoản thu nhập tương tự",income_statement!$A:$A,0),MATCH(I$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J53" s="19" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="20" t="inlineStr">
+        <is>
+          <t>Chi phí lãi</t>
+        </is>
+      </c>
+      <c r="B54" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Chi phí lãi và các chi phí tương tự",income_statement!$A:$A,0),MATCH(B$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C54" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Chi phí lãi và các chi phí tương tự",income_statement!$A:$A,0),MATCH(C$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D54" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Chi phí lãi và các chi phí tương tự",income_statement!$A:$A,0),MATCH(D$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E54" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Chi phí lãi và các chi phí tương tự",income_statement!$A:$A,0),MATCH(E$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="F54" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Chi phí lãi và các chi phí tương tự",income_statement!$A:$A,0),MATCH(F$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G54" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Chi phí lãi và các chi phí tương tự",income_statement!$A:$A,0),MATCH(G$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="H54" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Chi phí lãi và các chi phí tương tự",income_statement!$A:$A,0),MATCH(H$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="I54" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Chi phí lãi và các chi phí tương tự",income_statement!$A:$A,0),MATCH(I$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J54" s="19" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="16" t="inlineStr">
+        <is>
+          <t>Thu nhập lãi thuần</t>
+        </is>
+      </c>
+      <c r="B55" s="27">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Thu nhập lãi thuần",income_statement!$A:$A,0),MATCH(B$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C55" s="27">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Thu nhập lãi thuần",income_statement!$A:$A,0),MATCH(C$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D55" s="27">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Thu nhập lãi thuần",income_statement!$A:$A,0),MATCH(D$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E55" s="27">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Thu nhập lãi thuần",income_statement!$A:$A,0),MATCH(E$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="F55" s="27">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Thu nhập lãi thuần",income_statement!$A:$A,0),MATCH(F$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G55" s="27">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Thu nhập lãi thuần",income_statement!$A:$A,0),MATCH(G$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="H55" s="27">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Thu nhập lãi thuần",income_statement!$A:$A,0),MATCH(H$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="I55" s="27">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Thu nhập lãi thuần",income_statement!$A:$A,0),MATCH(I$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J55" s="31" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="20" t="inlineStr">
+        <is>
+          <t>Thu nhập ngoài lãi</t>
+        </is>
+      </c>
+      <c r="B56" s="25">
+        <f>IF(OR(B$57="",B$55=""),"",B$57-B$55)</f>
+        <v/>
+      </c>
+      <c r="C56" s="25">
+        <f>IF(OR(C$57="",C$55=""),"",C$57-C$55)</f>
+        <v/>
+      </c>
+      <c r="D56" s="25">
+        <f>IF(OR(D$57="",D$55=""),"",D$57-D$55)</f>
+        <v/>
+      </c>
+      <c r="E56" s="25">
+        <f>IF(OR(E$57="",E$55=""),"",E$57-E$55)</f>
+        <v/>
+      </c>
+      <c r="F56" s="25">
+        <f>IF(OR(F$57="",F$55=""),"",F$57-F$55)</f>
+        <v/>
+      </c>
+      <c r="G56" s="25">
+        <f>IF(OR(G$57="",G$55=""),"",G$57-G$55)</f>
+        <v/>
+      </c>
+      <c r="H56" s="25">
+        <f>IF(OR(H$57="",H$55=""),"",H$57-H$55)</f>
+        <v/>
+      </c>
+      <c r="I56" s="25">
+        <f>IF(OR(I$57="",I$55=""),"",I$57-I$55)</f>
+        <v/>
+      </c>
+      <c r="J56" s="19" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="20" t="inlineStr">
+        <is>
+          <t>Tổng thu nhập hoạt động</t>
+        </is>
+      </c>
+      <c r="B57" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Tổng thu nhập hoạt động",income_statement!$A:$A,0),MATCH(B$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C57" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Tổng thu nhập hoạt động",income_statement!$A:$A,0),MATCH(C$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D57" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Tổng thu nhập hoạt động",income_statement!$A:$A,0),MATCH(D$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E57" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Tổng thu nhập hoạt động",income_statement!$A:$A,0),MATCH(E$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="F57" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Tổng thu nhập hoạt động",income_statement!$A:$A,0),MATCH(F$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G57" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Tổng thu nhập hoạt động",income_statement!$A:$A,0),MATCH(G$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="H57" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Tổng thu nhập hoạt động",income_statement!$A:$A,0),MATCH(H$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="I57" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Tổng thu nhập hoạt động",income_statement!$A:$A,0),MATCH(I$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J57" s="19" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="20" t="inlineStr">
+        <is>
+          <t>Chi phí hoạt động</t>
+        </is>
+      </c>
+      <c r="B58" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Chi phí quản lý doanh nghiệp",income_statement!$A:$A,0),MATCH(B$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C58" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Chi phí quản lý doanh nghiệp",income_statement!$A:$A,0),MATCH(C$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D58" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Chi phí quản lý doanh nghiệp",income_statement!$A:$A,0),MATCH(D$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E58" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Chi phí quản lý doanh nghiệp",income_statement!$A:$A,0),MATCH(E$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="F58" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Chi phí quản lý doanh nghiệp",income_statement!$A:$A,0),MATCH(F$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G58" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Chi phí quản lý doanh nghiệp",income_statement!$A:$A,0),MATCH(G$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="H58" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Chi phí quản lý doanh nghiệp",income_statement!$A:$A,0),MATCH(H$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="I58" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Chi phí quản lý doanh nghiệp",income_statement!$A:$A,0),MATCH(I$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J58" s="19" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="20" t="inlineStr">
+        <is>
+          <t>Lãi và phí phải thu</t>
+        </is>
+      </c>
+      <c r="B59" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Các khoản lãi và phí phải thu",balance_sheet!$A:$A,0),MATCH(B$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C59" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Các khoản lãi và phí phải thu",balance_sheet!$A:$A,0),MATCH(C$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D59" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Các khoản lãi và phí phải thu",balance_sheet!$A:$A,0),MATCH(D$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E59" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Các khoản lãi và phí phải thu",balance_sheet!$A:$A,0),MATCH(E$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="F59" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Các khoản lãi và phí phải thu",balance_sheet!$A:$A,0),MATCH(F$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G59" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Các khoản lãi và phí phải thu",balance_sheet!$A:$A,0),MATCH(G$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="H59" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Các khoản lãi và phí phải thu",balance_sheet!$A:$A,0),MATCH(H$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="I59" s="21">
+        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Các khoản lãi và phí phải thu",balance_sheet!$A:$A,0),MATCH(I$21,balance_sheet!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J59" s="19" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="20" t="inlineStr">
+        <is>
+          <t>LNST</t>
+        </is>
+      </c>
+      <c r="B60" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Lợi nhuận sau thuế",income_statement!$A:$A,0),MATCH(B$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C60" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Lợi nhuận sau thuế",income_statement!$A:$A,0),MATCH(C$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D60" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Lợi nhuận sau thuế",income_statement!$A:$A,0),MATCH(D$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E60" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Lợi nhuận sau thuế",income_statement!$A:$A,0),MATCH(E$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="F60" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Lợi nhuận sau thuế",income_statement!$A:$A,0),MATCH(F$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G60" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Lợi nhuận sau thuế",income_statement!$A:$A,0),MATCH(G$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="H60" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Lợi nhuận sau thuế",income_statement!$A:$A,0),MATCH(H$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="I60" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Lợi nhuận sau thuế",income_statement!$A:$A,0),MATCH(I$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J60" s="19" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="20" t="inlineStr">
+        <is>
+          <t>LNST CĐ Công ty mẹ</t>
+        </is>
+      </c>
+      <c r="B61" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Cổ đông của Công ty mẹ",income_statement!$A:$A,0),MATCH(B$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C61" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Cổ đông của Công ty mẹ",income_statement!$A:$A,0),MATCH(C$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D61" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Cổ đông của Công ty mẹ",income_statement!$A:$A,0),MATCH(D$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E61" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Cổ đông của Công ty mẹ",income_statement!$A:$A,0),MATCH(E$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="F61" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Cổ đông của Công ty mẹ",income_statement!$A:$A,0),MATCH(F$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G61" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Cổ đông của Công ty mẹ",income_statement!$A:$A,0),MATCH(G$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="H61" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Cổ đông của Công ty mẹ",income_statement!$A:$A,0),MATCH(H$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="I61" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Cổ đông của Công ty mẹ",income_statement!$A:$A,0),MATCH(I$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J61" s="21" t="n">
+        <v>30415000000000</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="20" t="inlineStr">
+        <is>
+          <t>Tổng lợi nhuận/lỗ trước thuế</t>
+        </is>
+      </c>
+      <c r="B62" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Tổng lợi nhuận/lỗ trước thuế",income_statement!$A:$A,0),MATCH(B$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C62" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Tổng lợi nhuận/lỗ trước thuế",income_statement!$A:$A,0),MATCH(C$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D62" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Tổng lợi nhuận/lỗ trước thuế",income_statement!$A:$A,0),MATCH(D$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E62" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Tổng lợi nhuận/lỗ trước thuế",income_statement!$A:$A,0),MATCH(E$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="F62" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Tổng lợi nhuận/lỗ trước thuế",income_statement!$A:$A,0),MATCH(F$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G62" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Tổng lợi nhuận/lỗ trước thuế",income_statement!$A:$A,0),MATCH(G$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="H62" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Tổng lợi nhuận/lỗ trước thuế",income_statement!$A:$A,0),MATCH(H$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="I62" s="21">
+        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Tổng lợi nhuận/lỗ trước thuế",income_statement!$A:$A,0),MATCH(I$21,income_statement!$B$1:$I$1,0)),"")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="C2:I2">
+    <cfRule type="cellIs" priority="5" operator="lessThan" dxfId="0">
+      <formula>0.15</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="6" operator="greaterThanOrEqual" dxfId="1">
+      <formula>0.15</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C3:I4">
+    <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
+      <formula>0.1</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="greaterThan" dxfId="1">
+      <formula>0.15</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="17.5" customWidth="1" min="2" max="2"/>
+    <col width="10.125" customWidth="1" min="7" max="7"/>
+    <col width="8.875" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="32" t="n"/>
+      <c r="B1" s="32" t="inlineStr">
+        <is>
+          <t>Q4/2025</t>
+        </is>
+      </c>
+      <c r="C1" s="32" t="inlineStr">
+        <is>
+          <t>Q1/2026</t>
+        </is>
+      </c>
+      <c r="D1" s="32" t="inlineStr">
+        <is>
+          <t>Q2/2026</t>
+        </is>
+      </c>
+      <c r="E1" s="32" t="inlineStr">
+        <is>
+          <t>Q3/2026</t>
+        </is>
+      </c>
+      <c r="F1" s="32" t="inlineStr">
+        <is>
+          <t>Q4/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="32" t="inlineStr">
+        <is>
+          <t>Số CP</t>
+        </is>
+      </c>
+      <c r="B2" s="33" t="n">
+        <v>8054999909</v>
+      </c>
+      <c r="C2" s="33" t="n">
+        <v>8054999909</v>
+      </c>
+      <c r="D2" s="33" t="n">
+        <v>8054999909</v>
+      </c>
+      <c r="E2" s="33" t="n">
+        <v>8054999909</v>
+      </c>
+      <c r="F2" s="33" t="n">
+        <v>8054999909</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="32" t="inlineStr">
+        <is>
+          <t>Thị giá</t>
+        </is>
+      </c>
+      <c r="B3" s="33" t="n">
+        <v>75100</v>
+      </c>
+      <c r="C3" s="33" t="n">
+        <v>75100</v>
+      </c>
+      <c r="D3" s="33" t="n">
+        <v>75100</v>
+      </c>
+      <c r="E3" s="33" t="n">
+        <v>75100</v>
+      </c>
+      <c r="F3" s="33" t="n">
+        <v>75100</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="32" t="inlineStr">
+        <is>
+          <t>Vốn hoá</t>
+        </is>
+      </c>
+      <c r="B4" s="33">
+        <f>B2*B3</f>
+        <v/>
+      </c>
+      <c r="C4" s="33">
+        <f>C2*C3</f>
+        <v/>
+      </c>
+      <c r="D4" s="33">
+        <f>D2*D3</f>
+        <v/>
+      </c>
+      <c r="E4" s="33">
+        <f>E2*E3</f>
+        <v/>
+      </c>
+      <c r="F4" s="33">
+        <f>F2*F3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5"/>
+    <row r="6">
+      <c r="A6" s="32" t="inlineStr">
+        <is>
+          <t>VCSH</t>
+        </is>
+      </c>
+      <c r="B6" s="33">
+        <f>chi_so_tai_chinh!I49</f>
+        <v/>
+      </c>
+      <c r="C6" s="33">
+        <f>B$6*(($F$6/$B$6)^(1/4))</f>
+        <v/>
+      </c>
+      <c r="D6" s="33">
+        <f>B$6*(($F$6/$B$6)^(2/4))</f>
+        <v/>
+      </c>
+      <c r="E6" s="33">
+        <f>B$6*(($F$6/$B$6)^(3/4))</f>
+        <v/>
+      </c>
+      <c r="F6" s="33">
+        <f>chi_so_tai_chinh!J49</f>
+        <v/>
+      </c>
+      <c r="G6" s="34" t="n"/>
+      <c r="H6" s="34" t="n"/>
+      <c r="I6" s="34" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="32" t="inlineStr">
+        <is>
+          <t>LICĐKKS</t>
+        </is>
+      </c>
+      <c r="B7" s="35">
+        <f>chi_so_tai_chinh!I51</f>
+        <v/>
+      </c>
+      <c r="C7" s="35">
+        <f>C6*0.05</f>
+        <v/>
+      </c>
+      <c r="D7" s="35">
+        <f>D6*0.05</f>
+        <v/>
+      </c>
+      <c r="E7" s="35">
+        <f>E6*0.05</f>
+        <v/>
+      </c>
+      <c r="F7" s="35">
+        <f>F6*0.05</f>
+        <v/>
+      </c>
+      <c r="G7" s="36" t="n"/>
+      <c r="H7" s="36" t="n"/>
+      <c r="I7" s="36" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="32" t="inlineStr">
+        <is>
+          <t>BV</t>
+        </is>
+      </c>
+      <c r="B8" s="37">
+        <f>B6-B7</f>
+        <v/>
+      </c>
+      <c r="C8" s="37">
+        <f>C6-C7</f>
+        <v/>
+      </c>
+      <c r="D8" s="37">
+        <f>D6-D7</f>
+        <v/>
+      </c>
+      <c r="E8" s="37">
+        <f>E6-E7</f>
+        <v/>
+      </c>
+      <c r="F8" s="37">
+        <f>F6-F7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="24" t="inlineStr">
+        <is>
+          <t>BVPS</t>
+        </is>
+      </c>
+      <c r="B9" s="38">
+        <f>B8/B2</f>
+        <v/>
+      </c>
+      <c r="C9" s="38">
+        <f>C8/C2</f>
+        <v/>
+      </c>
+      <c r="D9" s="38">
+        <f>D8/D2</f>
+        <v/>
+      </c>
+      <c r="E9" s="38">
+        <f>E8/E2</f>
+        <v/>
+      </c>
+      <c r="F9" s="38">
+        <f>F8/F2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="24" t="inlineStr">
+        <is>
+          <t>PB</t>
+        </is>
+      </c>
+      <c r="B10" s="39">
+        <f>$F$3/B9</f>
+        <v/>
+      </c>
+      <c r="C10" s="39">
+        <f>$F$3/C9</f>
+        <v/>
+      </c>
+      <c r="D10" s="39">
+        <f>$F$3/D9</f>
+        <v/>
+      </c>
+      <c r="E10" s="39">
+        <f>$F$3/E9</f>
+        <v/>
+      </c>
+      <c r="F10" s="39">
+        <f>$F$3/F9</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44.5" customWidth="1" min="1" max="1"/>
+    <col width="11.375" customWidth="1" min="2" max="2"/>
+    <col width="12.25" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="12.125" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="32" t="inlineStr">
         <is>
           <t>Chỉ tiêu</t>
         </is>
       </c>
-      <c r="B3" s="9">
-        <f>'balance_sheet'!B1</f>
-        <v/>
-      </c>
-      <c r="C3" s="9">
-        <f>'balance_sheet'!C1</f>
-        <v/>
-      </c>
-      <c r="D3" s="9">
-        <f>'balance_sheet'!D1</f>
-        <v/>
-      </c>
-      <c r="E3" s="9">
-        <f>'balance_sheet'!E1</f>
-        <v/>
-      </c>
-      <c r="F3" s="9">
-        <f>'balance_sheet'!F1</f>
-        <v/>
-      </c>
-      <c r="G3" s="9">
-        <f>'balance_sheet'!G1</f>
-        <v/>
-      </c>
-      <c r="H3" s="9">
-        <f>'balance_sheet'!H1</f>
-        <v/>
-      </c>
-      <c r="I3" s="9">
-        <f>'balance_sheet'!I1</f>
-        <v/>
-      </c>
+      <c r="B1" s="32" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C1" s="32" t="n">
+        <v>2023</v>
+      </c>
+      <c r="D1" s="32" t="n">
+        <v>2024</v>
+      </c>
+      <c r="E1" s="32" t="n">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="32" t="inlineStr">
+        <is>
+          <t>Lợi nhuận trước thuế kế hoạch</t>
+        </is>
+      </c>
+      <c r="B2" s="33" t="n">
+        <v>20300000</v>
+      </c>
+      <c r="C2" s="33" t="n">
+        <v>26138350</v>
+      </c>
+      <c r="D2" s="33" t="n">
+        <v>28410000</v>
+      </c>
+      <c r="E2" s="33" t="n">
+        <v>32000000</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="32" t="inlineStr">
+        <is>
+          <t>Lợi nhuận trước thuế thu nhập doanh nghiệp</t>
+        </is>
+      </c>
+      <c r="B3" s="33">
+        <f>chi_so_tai_chinh!F62/1000000</f>
+        <v/>
+      </c>
+      <c r="C3" s="33">
+        <f>chi_so_tai_chinh!G62/1000000</f>
+        <v/>
+      </c>
+      <c r="D3" s="33">
+        <f>chi_so_tai_chinh!H62/1000000</f>
+        <v/>
+      </c>
+      <c r="E3" s="33" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
-        <is>
-          <t>1. Khả năng sinh lời</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="11" t="inlineStr">
-        <is>
-          <t>ROE (LNST CĐ Cty mẹ / VCSH bình quân)</t>
-        </is>
-      </c>
-      <c r="B5" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="C5" s="13">
-        <f>IFERROR(C$47/((C$32+B$32)/2),"n/a")</f>
-        <v/>
-      </c>
-      <c r="D5" s="13">
-        <f>IFERROR(D$47/((D$32+C$32)/2),"n/a")</f>
-        <v/>
-      </c>
-      <c r="E5" s="13">
-        <f>IFERROR(E$47/((E$32+D$32)/2),"n/a")</f>
-        <v/>
-      </c>
-      <c r="F5" s="13">
-        <f>IFERROR(F$47/((F$32+E$32)/2),"n/a")</f>
-        <v/>
-      </c>
-      <c r="G5" s="13">
-        <f>IFERROR(G$47/((G$32+F$32)/2),"n/a")</f>
-        <v/>
-      </c>
-      <c r="H5" s="13">
-        <f>IFERROR(H$47/((H$32+G$32)/2),"n/a")</f>
-        <v/>
-      </c>
-      <c r="I5" s="13">
-        <f>IFERROR(I$47/((I$32+H$32)/2),"n/a")</f>
-        <v/>
-      </c>
-    </row>
+      <c r="A4" s="32" t="inlineStr">
+        <is>
+          <t>%thực hiện</t>
+        </is>
+      </c>
+      <c r="B4" s="40">
+        <f>B3/B2</f>
+        <v/>
+      </c>
+      <c r="C4" s="40">
+        <f>C3/C2</f>
+        <v/>
+      </c>
+      <c r="D4" s="40">
+        <f>D3/D2</f>
+        <v/>
+      </c>
+      <c r="E4" s="40" t="n"/>
+    </row>
+    <row r="5"/>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
-        <is>
-          <t>ROA (LNST / Tổng tài sản bình quân)</t>
-        </is>
-      </c>
-      <c r="B6" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="C6" s="13">
-        <f>IFERROR(C$46/((C$33+B$33)/2),"n/a")</f>
-        <v/>
-      </c>
-      <c r="D6" s="13">
-        <f>IFERROR(D$46/((D$33+C$33)/2),"n/a")</f>
-        <v/>
-      </c>
-      <c r="E6" s="13">
-        <f>IFERROR(E$46/((E$33+D$33)/2),"n/a")</f>
-        <v/>
-      </c>
-      <c r="F6" s="13">
-        <f>IFERROR(F$46/((F$33+E$33)/2),"n/a")</f>
-        <v/>
-      </c>
-      <c r="G6" s="13">
-        <f>IFERROR(G$46/((G$33+F$33)/2),"n/a")</f>
-        <v/>
-      </c>
-      <c r="H6" s="13">
-        <f>IFERROR(H$46/((H$33+G$33)/2),"n/a")</f>
-        <v/>
-      </c>
-      <c r="I6" s="13">
-        <f>IFERROR(I$46/((I$33+H$33)/2),"n/a")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="11" t="inlineStr">
-        <is>
-          <t>Tăng trưởng LN Cổ đông Cty mẹ</t>
-        </is>
-      </c>
-      <c r="B7" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="C7" s="13">
-        <f>IFERROR((C$47-B$47)/ABS(B$47),"n/a")</f>
-        <v/>
-      </c>
-      <c r="D7" s="13">
-        <f>IFERROR((D$47-C$47)/ABS(C$47),"n/a")</f>
-        <v/>
-      </c>
-      <c r="E7" s="13">
-        <f>IFERROR((E$47-D$47)/ABS(D$47),"n/a")</f>
-        <v/>
-      </c>
-      <c r="F7" s="13">
-        <f>IFERROR((F$47-E$47)/ABS(E$47),"n/a")</f>
-        <v/>
-      </c>
-      <c r="G7" s="13">
-        <f>IFERROR((G$47-F$47)/ABS(F$47),"n/a")</f>
-        <v/>
-      </c>
-      <c r="H7" s="13">
-        <f>IFERROR((H$47-G$47)/ABS(G$47),"n/a")</f>
-        <v/>
-      </c>
-      <c r="I7" s="13">
-        <f>IFERROR((I$47-H$47)/ABS(H$47),"n/a")</f>
-        <v/>
-      </c>
-    </row>
+      <c r="A6" s="32" t="inlineStr">
+        <is>
+          <t>Trung vị %thực hiện LN trước thuế</t>
+        </is>
+      </c>
+      <c r="B6" s="40">
+        <f>MEDIAN(B4:D4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7"/>
     <row r="8">
-      <c r="A8" s="11" t="inlineStr">
-        <is>
-          <t>Tăng trưởng Doanh thu thuần</t>
-        </is>
-      </c>
-      <c r="B8" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="C8" s="13">
-        <f>IFERROR((C$39-B$39)/ABS(B$39),"n/a")</f>
-        <v/>
-      </c>
-      <c r="D8" s="13">
-        <f>IFERROR((D$39-C$39)/ABS(C$39),"n/a")</f>
-        <v/>
-      </c>
-      <c r="E8" s="13">
-        <f>IFERROR((E$39-D$39)/ABS(D$39),"n/a")</f>
-        <v/>
-      </c>
-      <c r="F8" s="13">
-        <f>IFERROR((F$39-E$39)/ABS(E$39),"n/a")</f>
-        <v/>
-      </c>
-      <c r="G8" s="13">
-        <f>IFERROR((G$39-F$39)/ABS(F$39),"n/a")</f>
-        <v/>
-      </c>
-      <c r="H8" s="13">
-        <f>IFERROR((H$39-G$39)/ABS(G$39),"n/a")</f>
-        <v/>
-      </c>
-      <c r="I8" s="13">
-        <f>IFERROR((I$39-H$39)/ABS(H$39),"n/a")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="10" t="inlineStr">
-        <is>
-          <t>2. Biên lợi nhuận</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="11" t="inlineStr">
-        <is>
-          <t>Biên lợi nhuận gộp</t>
-        </is>
-      </c>
-      <c r="B10" s="13">
-        <f>IFERROR(B$41/B$39,"n/a")</f>
-        <v/>
-      </c>
-      <c r="C10" s="13">
-        <f>IFERROR(C$41/C$39,"n/a")</f>
-        <v/>
-      </c>
-      <c r="D10" s="13">
-        <f>IFERROR(D$41/D$39,"n/a")</f>
-        <v/>
-      </c>
-      <c r="E10" s="13">
-        <f>IFERROR(E$41/E$39,"n/a")</f>
-        <v/>
-      </c>
-      <c r="F10" s="13">
-        <f>IFERROR(F$41/F$39,"n/a")</f>
-        <v/>
-      </c>
-      <c r="G10" s="13">
-        <f>IFERROR(G$41/G$39,"n/a")</f>
-        <v/>
-      </c>
-      <c r="H10" s="13">
-        <f>IFERROR(H$41/H$39,"n/a")</f>
-        <v/>
-      </c>
-      <c r="I10" s="13">
-        <f>IFERROR(I$41/I$39,"n/a")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="11" t="inlineStr">
-        <is>
-          <t>Biên lợi nhuận ròng</t>
-        </is>
-      </c>
-      <c r="B11" s="13">
-        <f>IFERROR(B$46/B$39,"n/a")</f>
-        <v/>
-      </c>
-      <c r="C11" s="13">
-        <f>IFERROR(C$46/C$39,"n/a")</f>
-        <v/>
-      </c>
-      <c r="D11" s="13">
-        <f>IFERROR(D$46/D$39,"n/a")</f>
-        <v/>
-      </c>
-      <c r="E11" s="13">
-        <f>IFERROR(E$46/E$39,"n/a")</f>
-        <v/>
-      </c>
-      <c r="F11" s="13">
-        <f>IFERROR(F$46/F$39,"n/a")</f>
-        <v/>
-      </c>
-      <c r="G11" s="13">
-        <f>IFERROR(G$46/G$39,"n/a")</f>
-        <v/>
-      </c>
-      <c r="H11" s="13">
-        <f>IFERROR(H$46/H$39,"n/a")</f>
-        <v/>
-      </c>
-      <c r="I11" s="13">
-        <f>IFERROR(I$46/I$39,"n/a")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="10" t="inlineStr">
-        <is>
-          <t>3. Đòn bẩy tài chính</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="11" t="inlineStr">
-        <is>
-          <t>D/E (Nợ vay / Vốn chủ sở hữu)</t>
-        </is>
-      </c>
-      <c r="B13" s="14">
-        <f>IFERROR((B$37+B$38)/B$32,"n/a")</f>
-        <v/>
-      </c>
-      <c r="C13" s="14">
-        <f>IFERROR((C$37+C$38)/C$32,"n/a")</f>
-        <v/>
-      </c>
-      <c r="D13" s="14">
-        <f>IFERROR((D$37+D$38)/D$32,"n/a")</f>
-        <v/>
-      </c>
-      <c r="E13" s="14">
-        <f>IFERROR((E$37+E$38)/E$32,"n/a")</f>
-        <v/>
-      </c>
-      <c r="F13" s="14">
-        <f>IFERROR((F$37+F$38)/F$32,"n/a")</f>
-        <v/>
-      </c>
-      <c r="G13" s="14">
-        <f>IFERROR((G$37+G$38)/G$32,"n/a")</f>
-        <v/>
-      </c>
-      <c r="H13" s="14">
-        <f>IFERROR((H$37+H$38)/H$32,"n/a")</f>
-        <v/>
-      </c>
-      <c r="I13" s="14">
-        <f>IFERROR((I$37+I$38)/I$32,"n/a")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">     - Nợ vay dài hạn/Vốn chủ sở hữu</t>
-        </is>
-      </c>
-      <c r="B14" s="14">
-        <f>IFERROR(B$38/B$32,"n/a")</f>
-        <v/>
-      </c>
-      <c r="C14" s="14">
-        <f>IFERROR(C$38/C$32,"n/a")</f>
-        <v/>
-      </c>
-      <c r="D14" s="14">
-        <f>IFERROR(D$38/D$32,"n/a")</f>
-        <v/>
-      </c>
-      <c r="E14" s="14">
-        <f>IFERROR(E$38/E$32,"n/a")</f>
-        <v/>
-      </c>
-      <c r="F14" s="14">
-        <f>IFERROR(F$38/F$32,"n/a")</f>
-        <v/>
-      </c>
-      <c r="G14" s="14">
-        <f>IFERROR(G$38/G$32,"n/a")</f>
-        <v/>
-      </c>
-      <c r="H14" s="14">
-        <f>IFERROR(H$38/H$32,"n/a")</f>
-        <v/>
-      </c>
-      <c r="I14" s="14">
-        <f>IFERROR(I$38/I$32,"n/a")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">     - Nợ vay ngắn hạn/Vốn chủ sở hữu</t>
-        </is>
-      </c>
-      <c r="B15" s="14">
-        <f>IFERROR(B$37/B$32,"n/a")</f>
-        <v/>
-      </c>
-      <c r="C15" s="14">
-        <f>IFERROR(C$37/C$32,"n/a")</f>
-        <v/>
-      </c>
-      <c r="D15" s="14">
-        <f>IFERROR(D$37/D$32,"n/a")</f>
-        <v/>
-      </c>
-      <c r="E15" s="14">
-        <f>IFERROR(E$37/E$32,"n/a")</f>
-        <v/>
-      </c>
-      <c r="F15" s="14">
-        <f>IFERROR(F$37/F$32,"n/a")</f>
-        <v/>
-      </c>
-      <c r="G15" s="14">
-        <f>IFERROR(G$37/G$32,"n/a")</f>
-        <v/>
-      </c>
-      <c r="H15" s="14">
-        <f>IFERROR(H$37/H$32,"n/a")</f>
-        <v/>
-      </c>
-      <c r="I15" s="14">
-        <f>IFERROR(I$37/I$32,"n/a")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="11" t="inlineStr">
-        <is>
-          <t>Nợ phải trả/Vốn chủ sở hữu</t>
-        </is>
-      </c>
-      <c r="B16" s="14">
-        <f>IFERROR(B$34/B$32,"n/a")</f>
-        <v/>
-      </c>
-      <c r="C16" s="14">
-        <f>IFERROR(C$34/C$32,"n/a")</f>
-        <v/>
-      </c>
-      <c r="D16" s="14">
-        <f>IFERROR(D$34/D$32,"n/a")</f>
-        <v/>
-      </c>
-      <c r="E16" s="14">
-        <f>IFERROR(E$34/E$32,"n/a")</f>
-        <v/>
-      </c>
-      <c r="F16" s="14">
-        <f>IFERROR(F$34/F$32,"n/a")</f>
-        <v/>
-      </c>
-      <c r="G16" s="14">
-        <f>IFERROR(G$34/G$32,"n/a")</f>
-        <v/>
-      </c>
-      <c r="H16" s="14">
-        <f>IFERROR(H$34/H$32,"n/a")</f>
-        <v/>
-      </c>
-      <c r="I16" s="14">
-        <f>IFERROR(I$34/I$32,"n/a")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">     - Nợ dài hạn/Vốn chủ sở hữu</t>
-        </is>
-      </c>
-      <c r="B17" s="14">
-        <f>IFERROR(B$36/B$32,"n/a")</f>
-        <v/>
-      </c>
-      <c r="C17" s="14">
-        <f>IFERROR(C$36/C$32,"n/a")</f>
-        <v/>
-      </c>
-      <c r="D17" s="14">
-        <f>IFERROR(D$36/D$32,"n/a")</f>
-        <v/>
-      </c>
-      <c r="E17" s="14">
-        <f>IFERROR(E$36/E$32,"n/a")</f>
-        <v/>
-      </c>
-      <c r="F17" s="14">
-        <f>IFERROR(F$36/F$32,"n/a")</f>
-        <v/>
-      </c>
-      <c r="G17" s="14">
-        <f>IFERROR(G$36/G$32,"n/a")</f>
-        <v/>
-      </c>
-      <c r="H17" s="14">
-        <f>IFERROR(H$36/H$32,"n/a")</f>
-        <v/>
-      </c>
-      <c r="I17" s="14">
-        <f>IFERROR(I$36/I$32,"n/a")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">     - Nợ ngắn hạn/Vốn chủ sở hữu</t>
-        </is>
-      </c>
-      <c r="B18" s="14">
-        <f>IFERROR(B$35/B$32,"n/a")</f>
-        <v/>
-      </c>
-      <c r="C18" s="14">
-        <f>IFERROR(C$35/C$32,"n/a")</f>
-        <v/>
-      </c>
-      <c r="D18" s="14">
-        <f>IFERROR(D$35/D$32,"n/a")</f>
-        <v/>
-      </c>
-      <c r="E18" s="14">
-        <f>IFERROR(E$35/E$32,"n/a")</f>
-        <v/>
-      </c>
-      <c r="F18" s="14">
-        <f>IFERROR(F$35/F$32,"n/a")</f>
-        <v/>
-      </c>
-      <c r="G18" s="14">
-        <f>IFERROR(G$35/G$32,"n/a")</f>
-        <v/>
-      </c>
-      <c r="H18" s="14">
-        <f>IFERROR(H$35/H$32,"n/a")</f>
-        <v/>
-      </c>
-      <c r="I18" s="14">
-        <f>IFERROR(I$35/I$32,"n/a")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="10" t="inlineStr">
-        <is>
-          <t>4. Chi phí &amp; khả năng trả lãi</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="11" t="inlineStr">
-        <is>
-          <t>Chi phí bán hàng, quản lý/LN gộp</t>
-        </is>
-      </c>
-      <c r="B20" s="13">
-        <f>IFERROR((ABS(B$42)+ABS(B$43))/B$41,"n/a")</f>
-        <v/>
-      </c>
-      <c r="C20" s="13">
-        <f>IFERROR((ABS(C$42)+ABS(C$43))/C$41,"n/a")</f>
-        <v/>
-      </c>
-      <c r="D20" s="13">
-        <f>IFERROR((ABS(D$42)+ABS(D$43))/D$41,"n/a")</f>
-        <v/>
-      </c>
-      <c r="E20" s="13">
-        <f>IFERROR((ABS(E$42)+ABS(E$43))/E$41,"n/a")</f>
-        <v/>
-      </c>
-      <c r="F20" s="13">
-        <f>IFERROR((ABS(F$42)+ABS(F$43))/F$41,"n/a")</f>
-        <v/>
-      </c>
-      <c r="G20" s="13">
-        <f>IFERROR((ABS(G$42)+ABS(G$43))/G$41,"n/a")</f>
-        <v/>
-      </c>
-      <c r="H20" s="13">
-        <f>IFERROR((ABS(H$42)+ABS(H$43))/H$41,"n/a")</f>
-        <v/>
-      </c>
-      <c r="I20" s="13">
-        <f>IFERROR((ABS(I$42)+ABS(I$43))/I$41,"n/a")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="11" t="inlineStr">
-        <is>
-          <t>Chi phí lãi vay/LN từ hoạt động kinh doanh</t>
-        </is>
-      </c>
-      <c r="B21" s="13">
-        <f>IFERROR(ABS(B$45)/B$44,"n/a")</f>
-        <v/>
-      </c>
-      <c r="C21" s="13">
-        <f>IFERROR(ABS(C$45)/C$44,"n/a")</f>
-        <v/>
-      </c>
-      <c r="D21" s="13">
-        <f>IFERROR(ABS(D$45)/D$44,"n/a")</f>
-        <v/>
-      </c>
-      <c r="E21" s="13">
-        <f>IFERROR(ABS(E$45)/E$44,"n/a")</f>
-        <v/>
-      </c>
-      <c r="F21" s="13">
-        <f>IFERROR(ABS(F$45)/F$44,"n/a")</f>
-        <v/>
-      </c>
-      <c r="G21" s="13">
-        <f>IFERROR(ABS(G$45)/G$44,"n/a")</f>
-        <v/>
-      </c>
-      <c r="H21" s="13">
-        <f>IFERROR(ABS(H$45)/H$44,"n/a")</f>
-        <v/>
-      </c>
-      <c r="I21" s="13">
-        <f>IFERROR(ABS(I$45)/I$44,"n/a")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="10" t="inlineStr">
-        <is>
-          <t>5. Chu kỳ hoạt động vốn lưu động</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="11" t="inlineStr">
-        <is>
-          <t>Số ngày phải trả (DPO)</t>
-        </is>
-      </c>
-      <c r="B23" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="C23" s="15">
-        <f>IFERROR(((C$49+B$49)/2)/ABS(C$40)*365,"n/a")</f>
-        <v/>
-      </c>
-      <c r="D23" s="15">
-        <f>IFERROR(((D$49+C$49)/2)/ABS(D$40)*365,"n/a")</f>
-        <v/>
-      </c>
-      <c r="E23" s="15">
-        <f>IFERROR(((E$49+D$49)/2)/ABS(E$40)*365,"n/a")</f>
-        <v/>
-      </c>
-      <c r="F23" s="15">
-        <f>IFERROR(((F$49+E$49)/2)/ABS(F$40)*365,"n/a")</f>
-        <v/>
-      </c>
-      <c r="G23" s="15">
-        <f>IFERROR(((G$49+F$49)/2)/ABS(G$40)*365,"n/a")</f>
-        <v/>
-      </c>
-      <c r="H23" s="15">
-        <f>IFERROR(((H$49+G$49)/2)/ABS(H$40)*365,"n/a")</f>
-        <v/>
-      </c>
-      <c r="I23" s="15">
-        <f>IFERROR(((I$49+H$49)/2)/ABS(I$40)*365,"n/a")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="11" t="inlineStr">
-        <is>
-          <t>Số ngày phải thu (DSO)</t>
-        </is>
-      </c>
-      <c r="B24" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="C24" s="15">
-        <f>IFERROR(((C$48+B$48)/2)/C$39*365,"n/a")</f>
-        <v/>
-      </c>
-      <c r="D24" s="15">
-        <f>IFERROR(((D$48+C$48)/2)/D$39*365,"n/a")</f>
-        <v/>
-      </c>
-      <c r="E24" s="15">
-        <f>IFERROR(((E$48+D$48)/2)/E$39*365,"n/a")</f>
-        <v/>
-      </c>
-      <c r="F24" s="15">
-        <f>IFERROR(((F$48+E$48)/2)/F$39*365,"n/a")</f>
-        <v/>
-      </c>
-      <c r="G24" s="15">
-        <f>IFERROR(((G$48+F$48)/2)/G$39*365,"n/a")</f>
-        <v/>
-      </c>
-      <c r="H24" s="15">
-        <f>IFERROR(((H$48+G$48)/2)/H$39*365,"n/a")</f>
-        <v/>
-      </c>
-      <c r="I24" s="15">
-        <f>IFERROR(((I$48+H$48)/2)/I$39*365,"n/a")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="11" t="inlineStr">
-        <is>
-          <t>Số ngày tồn kho (DIO)</t>
-        </is>
-      </c>
-      <c r="B25" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="C25" s="15">
-        <f>IFERROR(((C$50+B$50)/2)/ABS(C$40)*365,"n/a")</f>
-        <v/>
-      </c>
-      <c r="D25" s="15">
-        <f>IFERROR(((D$50+C$50)/2)/ABS(D$40)*365,"n/a")</f>
-        <v/>
-      </c>
-      <c r="E25" s="15">
-        <f>IFERROR(((E$50+D$50)/2)/ABS(E$40)*365,"n/a")</f>
-        <v/>
-      </c>
-      <c r="F25" s="15">
-        <f>IFERROR(((F$50+E$50)/2)/ABS(F$40)*365,"n/a")</f>
-        <v/>
-      </c>
-      <c r="G25" s="15">
-        <f>IFERROR(((G$50+F$50)/2)/ABS(G$40)*365,"n/a")</f>
-        <v/>
-      </c>
-      <c r="H25" s="15">
-        <f>IFERROR(((H$50+G$50)/2)/ABS(H$40)*365,"n/a")</f>
-        <v/>
-      </c>
-      <c r="I25" s="15">
-        <f>IFERROR(((I$50+H$50)/2)/ABS(I$40)*365,"n/a")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="10" t="inlineStr">
-        <is>
-          <t>6. Cơ cấu tài sản</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="11" t="inlineStr">
-        <is>
-          <t>Tiền và tương đương tiền/Tài sản</t>
-        </is>
-      </c>
-      <c r="B27" s="13">
-        <f>IFERROR(B$51/B$33,"n/a")</f>
-        <v/>
-      </c>
-      <c r="C27" s="13">
-        <f>IFERROR(C$51/C$33,"n/a")</f>
-        <v/>
-      </c>
-      <c r="D27" s="13">
-        <f>IFERROR(D$51/D$33,"n/a")</f>
-        <v/>
-      </c>
-      <c r="E27" s="13">
-        <f>IFERROR(E$51/E$33,"n/a")</f>
-        <v/>
-      </c>
-      <c r="F27" s="13">
-        <f>IFERROR(F$51/F$33,"n/a")</f>
-        <v/>
-      </c>
-      <c r="G27" s="13">
-        <f>IFERROR(G$51/G$33,"n/a")</f>
-        <v/>
-      </c>
-      <c r="H27" s="13">
-        <f>IFERROR(H$51/H$33,"n/a")</f>
-        <v/>
-      </c>
-      <c r="I27" s="13">
-        <f>IFERROR(I$51/I$33,"n/a")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="11" t="inlineStr">
-        <is>
-          <t>Hàng tồn kho/Tài sản</t>
-        </is>
-      </c>
-      <c r="B28" s="13">
-        <f>IFERROR(B$50/B$33,"n/a")</f>
-        <v/>
-      </c>
-      <c r="C28" s="13">
-        <f>IFERROR(C$50/C$33,"n/a")</f>
-        <v/>
-      </c>
-      <c r="D28" s="13">
-        <f>IFERROR(D$50/D$33,"n/a")</f>
-        <v/>
-      </c>
-      <c r="E28" s="13">
-        <f>IFERROR(E$50/E$33,"n/a")</f>
-        <v/>
-      </c>
-      <c r="F28" s="13">
-        <f>IFERROR(F$50/F$33,"n/a")</f>
-        <v/>
-      </c>
-      <c r="G28" s="13">
-        <f>IFERROR(G$50/G$33,"n/a")</f>
-        <v/>
-      </c>
-      <c r="H28" s="13">
-        <f>IFERROR(H$50/H$33,"n/a")</f>
-        <v/>
-      </c>
-      <c r="I28" s="13">
-        <f>IFERROR(I$50/I$33,"n/a")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29"/>
-    <row r="30">
-      <c r="A30" s="6" t="inlineStr">
-        <is>
-          <t>II. DỮ LIỆU TRÍCH XUẤT (tự động dò theo tên khoản mục)</t>
-        </is>
-      </c>
-      <c r="B30" s="7" t="n"/>
-      <c r="C30" s="7" t="n"/>
-      <c r="D30" s="7" t="n"/>
-      <c r="E30" s="7" t="n"/>
-      <c r="F30" s="7" t="n"/>
-      <c r="G30" s="7" t="n"/>
-      <c r="H30" s="7" t="n"/>
-      <c r="I30" s="7" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="8" t="inlineStr">
-        <is>
-          <t>Khoản mục</t>
-        </is>
-      </c>
-      <c r="B31" s="9">
-        <f>'balance_sheet'!B1</f>
-        <v/>
-      </c>
-      <c r="C31" s="9">
-        <f>'balance_sheet'!C1</f>
-        <v/>
-      </c>
-      <c r="D31" s="9">
-        <f>'balance_sheet'!D1</f>
-        <v/>
-      </c>
-      <c r="E31" s="9">
-        <f>'balance_sheet'!E1</f>
-        <v/>
-      </c>
-      <c r="F31" s="9">
-        <f>'balance_sheet'!F1</f>
-        <v/>
-      </c>
-      <c r="G31" s="9">
-        <f>'balance_sheet'!G1</f>
-        <v/>
-      </c>
-      <c r="H31" s="9">
-        <f>'balance_sheet'!H1</f>
-        <v/>
-      </c>
-      <c r="I31" s="9">
-        <f>'balance_sheet'!I1</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="3" t="inlineStr">
-        <is>
-          <t>VỐN CHỦ SỞ HỮU</t>
-        </is>
-      </c>
-      <c r="B32" s="16">
-        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("VỐN CHỦ SỞ HỮU",balance_sheet!$A:$A,0),MATCH(B$31,balance_sheet!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="C32" s="16">
-        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("VỐN CHỦ SỞ HỮU",balance_sheet!$A:$A,0),MATCH(C$31,balance_sheet!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="D32" s="16">
-        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("VỐN CHỦ SỞ HỮU",balance_sheet!$A:$A,0),MATCH(D$31,balance_sheet!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="E32" s="16">
-        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("VỐN CHỦ SỞ HỮU",balance_sheet!$A:$A,0),MATCH(E$31,balance_sheet!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="F32" s="16">
-        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("VỐN CHỦ SỞ HỮU",balance_sheet!$A:$A,0),MATCH(F$31,balance_sheet!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="G32" s="16">
-        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("VỐN CHỦ SỞ HỮU",balance_sheet!$A:$A,0),MATCH(G$31,balance_sheet!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="H32" s="16">
-        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("VỐN CHỦ SỞ HỮU",balance_sheet!$A:$A,0),MATCH(H$31,balance_sheet!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I32" s="16">
-        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("VỐN CHỦ SỞ HỮU",balance_sheet!$A:$A,0),MATCH(I$31,balance_sheet!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="3" t="inlineStr">
-        <is>
-          <t>TỔNG TÀI SẢN</t>
-        </is>
-      </c>
-      <c r="B33" s="16">
-        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("TỔNG TÀI SẢN",balance_sheet!$A:$A,0),MATCH(B$31,balance_sheet!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="C33" s="16">
-        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("TỔNG TÀI SẢN",balance_sheet!$A:$A,0),MATCH(C$31,balance_sheet!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="D33" s="16">
-        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("TỔNG TÀI SẢN",balance_sheet!$A:$A,0),MATCH(D$31,balance_sheet!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="E33" s="16">
-        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("TỔNG TÀI SẢN",balance_sheet!$A:$A,0),MATCH(E$31,balance_sheet!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="F33" s="16">
-        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("TỔNG TÀI SẢN",balance_sheet!$A:$A,0),MATCH(F$31,balance_sheet!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="G33" s="16">
-        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("TỔNG TÀI SẢN",balance_sheet!$A:$A,0),MATCH(G$31,balance_sheet!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="H33" s="16">
-        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("TỔNG TÀI SẢN",balance_sheet!$A:$A,0),MATCH(H$31,balance_sheet!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I33" s="16">
-        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("TỔNG TÀI SẢN",balance_sheet!$A:$A,0),MATCH(I$31,balance_sheet!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="3" t="inlineStr">
-        <is>
-          <t>TỔNG NỢ PHẢI TRẢ</t>
-        </is>
-      </c>
-      <c r="B34" s="16">
-        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("TỔNG NỢ PHẢI TRẢ",balance_sheet!$A:$A,0),MATCH(B$31,balance_sheet!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="C34" s="16">
-        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("TỔNG NỢ PHẢI TRẢ",balance_sheet!$A:$A,0),MATCH(C$31,balance_sheet!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="D34" s="16">
-        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("TỔNG NỢ PHẢI TRẢ",balance_sheet!$A:$A,0),MATCH(D$31,balance_sheet!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="E34" s="16">
-        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("TỔNG NỢ PHẢI TRẢ",balance_sheet!$A:$A,0),MATCH(E$31,balance_sheet!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="F34" s="16">
-        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("TỔNG NỢ PHẢI TRẢ",balance_sheet!$A:$A,0),MATCH(F$31,balance_sheet!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="G34" s="16">
-        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("TỔNG NỢ PHẢI TRẢ",balance_sheet!$A:$A,0),MATCH(G$31,balance_sheet!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="H34" s="16">
-        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("TỔNG NỢ PHẢI TRẢ",balance_sheet!$A:$A,0),MATCH(H$31,balance_sheet!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I34" s="16">
-        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("TỔNG NỢ PHẢI TRẢ",balance_sheet!$A:$A,0),MATCH(I$31,balance_sheet!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="3" t="inlineStr">
-        <is>
-          <t>Nợ ngắn hạn</t>
-        </is>
-      </c>
-      <c r="B35" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="C35" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="D35" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E35" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F35" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="G35" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H35" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="I35" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="3" t="inlineStr">
-        <is>
-          <t>Nợ dài hạn</t>
-        </is>
-      </c>
-      <c r="B36" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="C36" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="D36" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E36" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F36" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="G36" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H36" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="I36" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="3" t="inlineStr">
-        <is>
-          <t>Vay và nợ thuê tài chính ngắn hạn</t>
-        </is>
-      </c>
-      <c r="B37" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="C37" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="D37" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E37" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F37" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="G37" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H37" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="I37" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="3" t="inlineStr">
-        <is>
-          <t>Vay và nợ thuê tài chính dài hạn</t>
-        </is>
-      </c>
-      <c r="B38" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="C38" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="D38" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E38" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F38" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="G38" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H38" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="I38" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="3" t="inlineStr">
-        <is>
-          <t>Tổng thu nhập hoạt động</t>
-        </is>
-      </c>
-      <c r="B39" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Tổng thu nhập hoạt động",income_statement!$A:$A,0),MATCH(B$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="C39" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Tổng thu nhập hoạt động",income_statement!$A:$A,0),MATCH(C$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="D39" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Tổng thu nhập hoạt động",income_statement!$A:$A,0),MATCH(D$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="E39" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Tổng thu nhập hoạt động",income_statement!$A:$A,0),MATCH(E$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="F39" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Tổng thu nhập hoạt động",income_statement!$A:$A,0),MATCH(F$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="G39" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Tổng thu nhập hoạt động",income_statement!$A:$A,0),MATCH(G$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="H39" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Tổng thu nhập hoạt động",income_statement!$A:$A,0),MATCH(H$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I39" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Tổng thu nhập hoạt động",income_statement!$A:$A,0),MATCH(I$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="3" t="inlineStr">
-        <is>
-          <t>Giá vốn hàng bán / Chi phí hoạt động</t>
-        </is>
-      </c>
-      <c r="B40" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="C40" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="D40" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E40" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F40" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="G40" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H40" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="I40" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="3" t="inlineStr">
-        <is>
-          <t>Lợi nhuận gộp</t>
-        </is>
-      </c>
-      <c r="B41" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="C41" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="D41" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E41" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F41" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="G41" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H41" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="I41" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="3" t="inlineStr">
-        <is>
-          <t>Chi phí bán hàng</t>
-        </is>
-      </c>
-      <c r="B42" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="C42" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="D42" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E42" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F42" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="G42" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H42" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="I42" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="3" t="inlineStr">
-        <is>
-          <t>Chi phí quản lý doanh nghiệp</t>
-        </is>
-      </c>
-      <c r="B43" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Chi phí quản lý doanh nghiệp",income_statement!$A:$A,0),MATCH(B$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="C43" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Chi phí quản lý doanh nghiệp",income_statement!$A:$A,0),MATCH(C$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="D43" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Chi phí quản lý doanh nghiệp",income_statement!$A:$A,0),MATCH(D$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="E43" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Chi phí quản lý doanh nghiệp",income_statement!$A:$A,0),MATCH(E$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="F43" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Chi phí quản lý doanh nghiệp",income_statement!$A:$A,0),MATCH(F$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="G43" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Chi phí quản lý doanh nghiệp",income_statement!$A:$A,0),MATCH(G$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="H43" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Chi phí quản lý doanh nghiệp",income_statement!$A:$A,0),MATCH(H$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I43" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Chi phí quản lý doanh nghiệp",income_statement!$A:$A,0),MATCH(I$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="3" t="inlineStr">
-        <is>
-          <t>Lợi nhuận thuần hoạt động trước khi trích lập dự phòng tổn thất tín dụng</t>
-        </is>
-      </c>
-      <c r="B44" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Lợi nhuận thuần hoạt động trước khi trích lập dự phòng tổn thất tín dụng",income_statement!$A:$A,0),MATCH(B$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="C44" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Lợi nhuận thuần hoạt động trước khi trích lập dự phòng tổn thất tín dụng",income_statement!$A:$A,0),MATCH(C$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="D44" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Lợi nhuận thuần hoạt động trước khi trích lập dự phòng tổn thất tín dụng",income_statement!$A:$A,0),MATCH(D$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="E44" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Lợi nhuận thuần hoạt động trước khi trích lập dự phòng tổn thất tín dụng",income_statement!$A:$A,0),MATCH(E$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="F44" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Lợi nhuận thuần hoạt động trước khi trích lập dự phòng tổn thất tín dụng",income_statement!$A:$A,0),MATCH(F$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="G44" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Lợi nhuận thuần hoạt động trước khi trích lập dự phòng tổn thất tín dụng",income_statement!$A:$A,0),MATCH(G$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="H44" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Lợi nhuận thuần hoạt động trước khi trích lập dự phòng tổn thất tín dụng",income_statement!$A:$A,0),MATCH(H$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I44" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Lợi nhuận thuần hoạt động trước khi trích lập dự phòng tổn thất tín dụng",income_statement!$A:$A,0),MATCH(I$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="3" t="inlineStr">
-        <is>
-          <t>Chi phí lãi và các chi phí tương tự</t>
-        </is>
-      </c>
-      <c r="B45" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Chi phí lãi và các chi phí tương tự",income_statement!$A:$A,0),MATCH(B$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="C45" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Chi phí lãi và các chi phí tương tự",income_statement!$A:$A,0),MATCH(C$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="D45" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Chi phí lãi và các chi phí tương tự",income_statement!$A:$A,0),MATCH(D$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="E45" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Chi phí lãi và các chi phí tương tự",income_statement!$A:$A,0),MATCH(E$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="F45" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Chi phí lãi và các chi phí tương tự",income_statement!$A:$A,0),MATCH(F$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="G45" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Chi phí lãi và các chi phí tương tự",income_statement!$A:$A,0),MATCH(G$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="H45" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Chi phí lãi và các chi phí tương tự",income_statement!$A:$A,0),MATCH(H$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I45" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Chi phí lãi và các chi phí tương tự",income_statement!$A:$A,0),MATCH(I$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="3" t="inlineStr">
-        <is>
-          <t>Lợi nhuận sau thuế</t>
-        </is>
-      </c>
-      <c r="B46" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Lợi nhuận sau thuế",income_statement!$A:$A,0),MATCH(B$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="C46" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Lợi nhuận sau thuế",income_statement!$A:$A,0),MATCH(C$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="D46" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Lợi nhuận sau thuế",income_statement!$A:$A,0),MATCH(D$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="E46" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Lợi nhuận sau thuế",income_statement!$A:$A,0),MATCH(E$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="F46" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Lợi nhuận sau thuế",income_statement!$A:$A,0),MATCH(F$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="G46" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Lợi nhuận sau thuế",income_statement!$A:$A,0),MATCH(G$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="H46" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Lợi nhuận sau thuế",income_statement!$A:$A,0),MATCH(H$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I46" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Lợi nhuận sau thuế",income_statement!$A:$A,0),MATCH(I$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="3" t="inlineStr">
-        <is>
-          <t>Cổ đông của Công ty mẹ</t>
-        </is>
-      </c>
-      <c r="B47" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Cổ đông của Công ty mẹ",income_statement!$A:$A,0),MATCH(B$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="C47" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Cổ đông của Công ty mẹ",income_statement!$A:$A,0),MATCH(C$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="D47" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Cổ đông của Công ty mẹ",income_statement!$A:$A,0),MATCH(D$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="E47" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Cổ đông của Công ty mẹ",income_statement!$A:$A,0),MATCH(E$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="F47" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Cổ đông của Công ty mẹ",income_statement!$A:$A,0),MATCH(F$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="G47" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Cổ đông của Công ty mẹ",income_statement!$A:$A,0),MATCH(G$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="H47" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Cổ đông của Công ty mẹ",income_statement!$A:$A,0),MATCH(H$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I47" s="16">
-        <f>IFERROR(INDEX(income_statement!$B:$I,MATCH("Cổ đông của Công ty mẹ",income_statement!$A:$A,0),MATCH(I$31,income_statement!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="3" t="inlineStr">
-        <is>
-          <t>Phải thu khách hàng</t>
-        </is>
-      </c>
-      <c r="B48" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="C48" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="D48" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E48" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F48" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="G48" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H48" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="I48" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="3" t="inlineStr">
-        <is>
-          <t>Phải trả người bán</t>
-        </is>
-      </c>
-      <c r="B49" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="C49" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="D49" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E49" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F49" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="G49" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H49" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="I49" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="3" t="inlineStr">
-        <is>
-          <t>Hàng tồn kho, ròng</t>
-        </is>
-      </c>
-      <c r="B50" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="C50" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="D50" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="E50" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F50" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="G50" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H50" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="I50" s="12" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="3" t="inlineStr">
-        <is>
-          <t>Tiền mặt, vàng bạc, đá quý</t>
-        </is>
-      </c>
-      <c r="B51" s="16">
-        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Tiền mặt, vàng bạc, đá quý",balance_sheet!$A:$A,0),MATCH(B$31,balance_sheet!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="C51" s="16">
-        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Tiền mặt, vàng bạc, đá quý",balance_sheet!$A:$A,0),MATCH(C$31,balance_sheet!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="D51" s="16">
-        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Tiền mặt, vàng bạc, đá quý",balance_sheet!$A:$A,0),MATCH(D$31,balance_sheet!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="E51" s="16">
-        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Tiền mặt, vàng bạc, đá quý",balance_sheet!$A:$A,0),MATCH(E$31,balance_sheet!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="F51" s="16">
-        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Tiền mặt, vàng bạc, đá quý",balance_sheet!$A:$A,0),MATCH(F$31,balance_sheet!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="G51" s="16">
-        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Tiền mặt, vàng bạc, đá quý",balance_sheet!$A:$A,0),MATCH(G$31,balance_sheet!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="H51" s="16">
-        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Tiền mặt, vàng bạc, đá quý",balance_sheet!$A:$A,0),MATCH(H$31,balance_sheet!$B$1:$I$1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="I51" s="16">
-        <f>IFERROR(INDEX(balance_sheet!$B:$I,MATCH("Tiền mặt, vàng bạc, đá quý",balance_sheet!$A:$A,0),MATCH(I$31,balance_sheet!$B$1:$I$1,0)),"")</f>
+      <c r="A8" s="32" t="inlineStr">
+        <is>
+          <t>Tỷ lệ hoàn thành LNST trên 95%</t>
+        </is>
+      </c>
+      <c r="B8" s="40">
+        <f>COUNTIF(B4:D4,"&gt;=95%")/COUNT(B4:D4)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:I1"/>
-  </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="cellIs" priority="2" operator="greaterThanOrEqual" dxfId="1">
+      <formula>1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B8">
+    <cfRule type="cellIs" priority="1" operator="greaterThanOrEqual" dxfId="1">
+      <formula>1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B4:E4">
+    <cfRule type="cellIs" priority="3" operator="greaterThanOrEqual" dxfId="1">
+      <formula>1</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>